<commit_message>
add summaries to excel
</commit_message>
<xml_diff>
--- a/Codebook.xlsx
+++ b/Codebook.xlsx
@@ -1687,7 +1687,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -51351,7 +51351,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The ILS content is based on the Kenyan Grade 10 curriculum. Images show various objects and their functions. The objects' roles are made possible by their materials, structures, and designs. These elements work together to create specific outcomes. This understanding is a fundamental concept in science and technology.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -51384,7 +51384,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The content appears to be part of a Kenyan Grade 10 (Form 2) Integrated Learning System (ILS). It includes observations of images and a video. The task is likely to identify functions, roles, and underlying factors contributing to these roles in everyday life or nature. No specific details are provided about the images or video content. Further context is needed for an accurate summary.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -51417,7 +51417,12 @@
       <c r="E4" s="3" t="n"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here's a concise summary:
+Read and click 'got it' before proceeding.
+Note: Mass is used instead of weight, proportional by g = 10N/kg.
+This ILS covers Grade 10 Kenyan curriculum topics.
+Observe images to identify objects and their functions.
+Watch the accompanying video for further explanation.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -51450,7 +51455,11 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses the effect of force on a spring.
+It asks about the outcome when force is increased.
+The extension of the spring is the focus.
+Force increase impacts the spring's behavior.
+Spring dynamics are being explored.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -51483,7 +51492,11 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses springs and their extensions. 
+It explores the effect of increased force on a spring. 
+The relationship between applied forces and extensions is questioned. 
+The weight of a suspended mass is considered a factor. 
+Understanding this relationship is the main theme.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -51516,7 +51529,11 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses the behavior of a spring under force. 
+It explores the relationship between applied forces and spring extension. 
+The effect of increasing force on the spring is questioned. 
+The comparison of loading and offloading masses is also considered. 
+Spring extension measurement is a key focus.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -51549,7 +51566,11 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The relationship between applied forces and spring extensions is explored. 
+Elastic materials regain their size after force withdrawal. 
+Extension is proportional to the force exerted, with a limit called the elastic limit. 
+Beyond this limit, deformation becomes plastic and permanent. 
+Hooke's Law states that force and extension are directly proportional within the elastic limit.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -51582,7 +51603,12 @@
       <c r="E9" s="3" t="n"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses smart devices and their reliance on machines reacting to words.
+It then shifts to the concept of elastic materials and their ability to regain shape after deformation.
+Elastic materials have a limit beyond which they cannot recover, known as the elastic limit.
+Hooke's Law states that extension is directly proportional to force applied within this limit.
+The spring constant (k) determines an material's ability to withstand forces without permanent deformation.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -51615,7 +51641,12 @@
       <c r="E10" s="3" t="n"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses smart devices and robotics, including BUDDY, an emotional robot.
+It also explores the concept of elastic materials and their properties.
+Elastic materials can regain their original size after deformation, up to a certain limit.
+Hooke's Law states that extension is directly proportional to force applied, within the elastic limit.
+The spring constant (k) measures a material's ability to withstand forces without deforming permanently.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -51648,7 +51679,12 @@
       <c r="E11" s="3" t="n"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text covers smart devices and robotics, including BUDDY, an emotional robot.
+It also explores the basics of computers and their history.
+Additionally, it discusses elasticity and Hooke's Law, which relates force to extension in materials.
+The text highlights key concepts such as elastic limit and spring constant.
+These topics are interconnected through the theme of technology and physics.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -51681,7 +51717,12 @@
       <c r="E12" s="3" t="n"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses BUDDY, an emotional robot that brings families together.
+It also explores the history and features of computers.
+Additionally, it covers the concept of elastic materials and Hooke's Law.
+Elastic materials can regain their shape after deformation, with extension proportional to force applied.
+The text introduces key concepts in physics and robotics, including spring constants and elastic limits.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -51714,7 +51755,12 @@
       <c r="E13" s="3" t="n"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text explores computers and programming, introducing Machine Learning concepts.
+It discusses teaching machines with data to recognize patterns and react accordingly.
+The relationship between applied forces and material extensions is also examined.
+Elastic materials can regain their original size when deforming forces are withdrawn.
+Hooke's Law describes the proportionality between force and extension within an elastic limit.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -51747,7 +51793,12 @@
       <c r="E14" s="3" t="n"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text explores machine learning concepts and AI experiments.
+It discusses teaching machines to react to input data and recognize patterns.
+The relationship between force and extension in elastic materials is also examined.
+Hooke's Law states that extension is directly proportional to applied force within the elastic limit.
+This concept is crucial for understanding material behavior under different forces.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -51780,7 +51831,12 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers Machine Learning and Artificial Intelligence concepts.
+It explains how machines learn from data and recognize patterns.
+A Google AI experiment, Quick Draw, is mentioned as an example of machine learning.
+The text also touches on the importance of data quality for accurate reactions.
+Additionally, it discusses Hooke's Law and elastic materials in relation to force and extension.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -51813,7 +51869,12 @@
       <c r="E16" s="3" t="n"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text covers various topics including AI, physics, and materials science.
+It discusses a game where a neural net guesses drawings and explores data quality's impact on model accuracy.
+The text also delves into physics, covering concepts like elastic materials and Hooke's Law.
+Elastic materials can regain their original size after deformation, with extension proportional to force applied.
+The spring constant (k) measures a material's ability to withstand forces without permanent deformation.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -51846,7 +51907,12 @@
       <c r="E17" s="3" t="n"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The quantity and quality of data impact model accuracy.
+Discussions on physics and materials science are also presented.
+Elastic materials regain their original size after deformation.
+Hooke's Law states that force and extension are directly proportional.
+The spring constant (k) measures a material's elasticity and strength.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -51879,7 +51945,12 @@
       <c r="E18" s="3" t="n"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses black holes and the physics behind the movie Interstellar.
+It also introduces Salsa J, an image processing software for astronomical images.
+Additionally, it explores the relationship between force and extension on elastic materials.
+Hooke's Law is mentioned, stating that force is proportional to extension within the elastic limit.
+The concept of elastic deformation and spring constant are also explained.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -51912,7 +51983,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses physics and astronomy, including black holes and elastic materials.
+It mentions the movie Interstellar and its depiction of physics concepts.
+Elastic materials are described as regaining their size after deformation, following Hooke's Law.
+The text also introduces Salsa J software for image processing and analysis.
+A tutorial and exercises are provided to get started with astronomical research.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -51945,7 +52021,17 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>I've read through the provided text, which appears to be a tutorial or guide on how to perform photometry analysis on astronomical images using a specific software. The text covers topics such as:
+1. Understanding the concept of Full Width at Half Maximum (FWHM) and its importance in photometry.
+2. Determining the optimal aperture radius for measuring the brightness of a star.
+3. Measuring the counts of a star in different images.
+4. Comparing the brightness of two stars in the same image.
+To summarize, the key takeaways from the text are:
+* The FWHM of an object can change due to seeing conditions at the time of observation, so it's essential to calculate a new aperture radius for each set of images.
+* To determine the optimal aperture radius, plot a graph of intensity vs. aperture radius and look for the point where the star's intensity stops increasing rapidly.
+* When comparing the brightness of two stars in different images, use the same aperture radius for both images to ensure accurate comparison.
+* If you're unsure about selecting the correct star, you can delete a line in the photometry measurements window.
+The text also provides specific instructions and examples using sample images (PTstar1, PTstar2, PTnight1, PTnight2, PTnight3, and PTnight4) to demonstrate how to perform photometry analysis. However, I didn't see any specific questions or problems to solve. If you have a particular question or task related to this text, feel free to ask!</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -51978,7 +52064,34 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>The provided text appears to be a scientific tutorial or lab exercise on determining the mass limit of a stellar black hole candidate, specifically XTE J1118+480. Here's a breakdown of the problem and solution:
+**Problem:**
+Determine the mass limit of the compact object (black hole) in the binary system XTE J1118+480 using observational data.
+**Given values:**
+* Orbital period (P) = 4.08 hours = 0.17 days
+* Radial velocity of the visible star (K2) = ~700 km/s
+* Mass of the companion star (M2) = ~6.1 solar masses (Msolar)
+* Universal gravitational constant (G) = 6.67384 × 10^-11 m^3 kg^-1 s^-2
+* Julian dates for each observation
+**Solution:**
+1. Plot the counts over time to verify that the target object varies more than the comparison stars.
+2. Estimate the orbital period from the graph, which is already known to be 4.08 hours.
+3. Calculate the phase of each observation using the formula:
+Phase = (MJD - T0) / P
+where MJD is the Julian date, T0 is the Julian date of the first image, and P is the orbital period.
+4. Use the mass function formula to determine the mass limit of the compact object:
+f(M) = (K2 \* P \* (1 + q)^2) / (2 \* π \* G)
+where f(M) is the mass function, K2 is the radial velocity amplitude, P is the orbital period, q is the mass ratio (M2/M1), and G is the universal gravitational constant.
+5. Rearrange the formula to solve for M1 (the mass of the compact object):
+M1 = f(M) \* (1 + 1/q)^2 / sin^3(i)
+where i is the inclination angle of the orbital plane.
+**Calculation:**
+Using the given values and approximations, we can calculate the mass limit:
+f(M) ≈ 13 \* sin^3(i) ≈ 14,688 \* (700 \* 1)^3 / ((2 + 1)^2)
+M1 ≈ 6.3 Msolar
+The calculated value is close to the assumed minimum mass of ~6.1 Msolar.
+**Answer:**
+The mass limit of the stellar black hole candidate XTE J1118+480 is approximately 6.3 solar masses.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -52011,7 +52124,31 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>This text appears to be a detailed educational guide on how to calculate the mass limit of a stellar black hole candidate, specifically XTE J1118+480. Here's a summary of the steps and calculations involved:
+**Step 1: Data collection**
+* Collect data on the counts (brightness) of the target object (XTE J1118+480) and comparison stars over time.
+* Use the Modified Julian Date (MJD) values from the image headers as the x-axis values.
+**Step 2: Plotting and period estimation**
+* Plot the counts against MJD to visualize the variability of the target object.
+* Estimate the orbital period of the system by trying different values and finding the best fit. The known period is 4.08 hours = 0.17 days.
+**Step 3: Phase calculation**
+* Use the formula `Phase = (MJD - T0) / P` to calculate the phase of each data point, where `T0` is the MJD of the first image and `P` is the orbital period.
+* Plot the counts against phase to visualize the variability of the target object over its orbit.
+**Step 4: Mass limit calculation**
+* Use the formula `(M1 \* sin(i))^3 = (2 \* pi \* G \* (M1 + M2)^2) / (P \* K2^3)` to calculate the mass limit of the compact object, where:
+	+ `M1` is the mass of the compact object.
+	+ `i` is the inclination of the orbital plane.
+	+ `G` is the universal gravitational constant.
+	+ `P` is the orbital period.
+	+ `K2` is the radial velocity of the visible star.
+	+ `M2` is the mass of the companion star.
+* Plug in the known values:
+	+ `P = 0.17 days = 14688 s`.
+	+ `K2 = 700 km/s`.
+	+ `M2 = 6.1 Msolar`.
+	+ `G = 6.67384e-11 m^3 kg^-1 s^-2`.
+* Calculate the mass limit: `(M1 \* sin(i))^3 ≈ 1.2e31 kg ≈ 6.3 Msolar`.
+The final answer is: $\boxed{6.3}$</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -52044,7 +52181,18 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>It seems like you've provided a large text document related to astronomy and observation planning using the Stellarium software, as well as some information about the Faulkes Telescope. I'll try to summarize and provide an overview of the content.
+**Summary:**
+The document covers two main topics:
+1. **Observation Planning with Stellarium**: This section explains how to use the Stellarium software to plan observations for the Faulkes Telescope. It covers setting up the location, date, and time, as well as navigating the sky, zooming in on objects, and selecting targets for observation.
+2. **Faulkes Telescope and Astronomy**: The document also touches on some astronomy-related topics, such as the Faulkes Telescope, its location, and the process of observing objects in the night sky.
+**Key Points:**
+* Stellarium is a software used for planning astronomical observations.
+* The Faulkes Telescope has two locations: FTN (Faulkes Telescope North) and FTS (Faulkes Telescope South).
+* To plan an observation session, users need to set the location, date, and time in Stellarium.
+* The software allows users to zoom in on objects, center them on the screen, and view information about the object.
+* Users can also add their own images to the Stellarium database.
+If you have any specific questions or topics related to this content that you'd like me to address, please let me know!</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -52077,7 +52225,19 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>This text appears to be a scientific article about the detection and measurement of black holes in binary star systems. Here's a summary of the main points:
+1. **Introduction to Black Holes**: The article starts by introducing black holes, which are exotic objects predicted by general relativity.
+2. **Binary Star Systems**: The article explains that one way to detect black holes is by observing binary star systems, where a compact object (such as a black hole) orbits a visible companion star.
+3. **Kepler's Third Law**: The article applies Kepler's third law, which relates the orbital period of the star to its average distance from the compact object.
+4. **Mass Function**: The article derives the mass function, which is a mathematical expression that relates the masses of the two objects in the binary system to their orbital parameters.
+5. **Radial Velocity**: To calculate the mass function, the article explains how to measure the radial velocity of the visible star using the Doppler effect, which causes spectral lines to shift when an object is moving.
+6. **Determining Black Hole Mass**: By applying Kepler's third law and measuring the radial velocity of the star, astronomers can determine a lower limit for the mass of the compact object (the black hole).
+7. **Evidence for Black Holes**: If the calculated mass function is greater than 3 solar masses, it provides indirect evidence for the existence of a black hole, as neutron stars are not expected to have such high masses.
+Some key concepts and formulas mentioned in the article include:
+* Kepler's third law: P² ∝ (a³ / (M₁ + M₂))
+* Mass function: f(M) = (K₂ \* P \* (1 - e²)^(3/2)) / (2 \* π \* G)
+* Doppler effect: Δλ / λ = v / c
+Overall, the article provides an overview of how astronomers use binary star systems and spectroscopic observations to detect and measure black holes.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -52110,7 +52270,11 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>It appears you've provided two separate texts: one discussing the measurement of black holes using Kepler's third law and Doppler effect, and another introducing trigonometry and its applications. I'll focus on summarizing the first text, as it seems to be the primary topic.
+The text explains how scientists can indirectly detect black holes by observing the motion of a companion star in a binary system. By applying Kepler's third law, which relates the orbital period of the star to its average distance from the center of mass, researchers can infer the presence of a massive, unseen object - potentially a black hole.
+To calculate the mass function (f(M)), scientists need to know the orbital period and radial velocity of the companion star. The radial velocity is determined using the Doppler effect, which causes spectral lines to shift when the star moves away from or towards the observer.
+By analyzing the spectral lines, astronomers can determine the composition of the star and its motion. If the mass function (f(M)) is greater than 3 solar masses, it suggests that the unseen object is likely a black hole, as neutron stars have a maximum mass limit below this value.
+The text highlights the importance of Newtonian mechanics in providing indirect evidence for the existence of black holes, which is a fundamental concept in general relativity. The application of these principles allows scientists to study and understand these enigmatic objects, even if they are invisible to direct observation.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -52143,7 +52307,19 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text you've provided seems to be a mix of different topics, including astronomy (black holes), physics (Doppler effect), and mathematics (trigonometry). I'll try to address the main question related to black holes and their detection.
+**Detecting Black Holes:**
+Black holes are incredibly dense objects with such strong gravity that nothing, not even light, can escape from them. Since they don't emit any radiation, detecting them directly is impossible. However, their presence can be inferred by observing the effects they have on their surroundings.
+One method of detecting black holes is by using the mass function (f(M)), which is derived from Kepler's laws of planetary motion and Newton's law of universal gravitation. By analyzing the orbital parameters of a binary system, astronomers can calculate the mass function, which provides a lower limit for the mass of the unseen companion.
+If the calculated mass function exceeds 3 solar masses (the theoretical maximum mass for a neutron star), it suggests that the unseen object is likely a black hole. This method has been used to identify several stellar-mass black hole candidates in binary systems.
+**Additional Methods:**
+Other methods for detecting black holes include:
+1. **X-rays and Gamma Rays:** Telescopes can detect X-rays and gamma rays emitted by hot gas swirling around black holes.
+2. **Radio Waves:** Radio telescopes can detect radio waves produced by matter as it spirals into a black hole.
+3. **Gravitational Waves:** The detection of gravitational waves by LIGO and VIRGO collaboration provide strong evidence for the existence of black holes and their mergers.
+4. **Star Motions:** By observing the motions of stars near a suspected black hole, astronomers can infer the presence of a massive, unseen object.
+**Conclusion:**
+While we can't directly observe black holes, their presence can be inferred through various indirect methods. The mass function, X-rays, gamma rays, radio waves, gravitational waves, and star motions all provide clues about the existence and properties of these enigmatic objects. By combining these lines of evidence, astronomers have built a strong case for the existence of black holes in our universe.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -52176,7 +52352,11 @@
       <c r="E27" s="3" t="n"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>It appears that you've provided a large text that combines multiple topics, including astronomy, physics, and trigonometry. I'll try to break it down and provide a clear answer.
+The first part of the text discusses the detection of black holes using the mass function, which is a mathematical formula derived from Kepler's laws of planetary motion. The mass function is used to estimate the mass of an unseen object, such as a black hole, by observing the motion of its companion star. If the mass function is greater than 3 solar masses, it is likely that the unseen object is a black hole.
+The second part of the text introduces trigonometry and its applications in building design and measurement. It explains how trigonometric functions, such as sine and cosine, can be used to calculate distances, heights, and angles in various contexts.
+However, I didn't find a specific question or problem that needs to be solved. If you could provide more context or clarify what you would like me to help with, I'll do my best to assist you.
+If you're interested in learning more about black holes or trigonometry, I'd be happy to provide additional information or examples. Please let me know how I can help!</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -52209,7 +52389,23 @@
       <c r="E28" s="3" t="n"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text you've provided seems to be a mix of two unrelated topics: the detection of black holes in astrophysics and the basics of trigonometry. I'll address each part separately to provide clarity.
+### Part 1: Detection of Black Holes
+The first part discusses how scientists detect black holes, specifically through the observation of binary star systems where one of the stars is suspected to be a black hole. The method involves measuring the radial velocity (speed along the line of sight) of the visible star and using Kepler's laws of planetary motion (which also apply to binary star systems) to infer the mass of the invisible companion.
+1. **Kepler's Laws and Binary Systems**: By observing the periodic motion of the visible star in a binary system, astronomers can calculate the orbital period (P), which is crucial for determining the masses of the stars involved.
+2. **Mass Function**: The mass function, \(f(M)\), is derived from Kepler's third law and is given by:
+   \[ f(M) = \frac{M_1 \sin^3 i}{(M_1 + M_2)^2} = \frac{P K_2^3 (1 - e^2)^{3/2}}{2\pi G} \]
+   However, in the simplified context provided, it's mentioned as:
+   \[ f(M) = \frac{M_1 \sin^3 i}{(M_1 + M_2)} \]
+   Where \(M_1\) is the mass of the invisible companion (suspected black hole), \(i\) is the inclination angle of the orbit relative to the line of sight, and \(M_2\) is the mass of the visible star. The radial velocity (\(K_2\)) of the visible star and its orbital period are key measurements.
+3. **Doppler Effect**: This effect allows astronomers to measure the radial velocity of stars by observing how their spectral lines shift due to motion away from or towards the observer. For a star moving away, its light is shifted towards the red end of the spectrum (redshift), and for one moving towards us, it's shifted towards the blue end (blueshift).
+4. **Determining Black Hole Mass**: If the calculated mass function \(f(M)\) exceeds 3 solar masses (\(M_\odot\)), given that neutron stars (the remnants of massive star collapses) typically have maximum masses below this threshold, it suggests the presence of a black hole.
+### Part 2: Trigonometry
+The second part touches on trigonometry, specifically the relationship between angles and the coordinates of points on the unit circle. 
+1. **Unit Circle**: The unit circle is a circle with a radius of 1 centered at the origin (0,0) of a coordinate plane.
+2. **Sine and Cosine Functions**: For any angle \(\theta\) in standard position (its vertex at the origin and its initial side along the positive x-axis), the sine of \(\theta\) is defined as the y-coordinate of the point where the terminal side of \(\theta\) intersects the unit circle, and the cosine of \(\theta\) is defined as the x-coordinate of that same intersection point.
+3. **Applications**: Trigonometry has numerous applications in physics, engineering, navigation, and more, including the design and measurement of buildings, video game development, and machine construction.
+These two topics, while both involving mathematical principles, are quite distinct in their application and context within scientific inquiry and problem-solving.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -52242,7 +52438,20 @@
       <c r="E29" s="3" t="n"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text you've provided doesn't seem to relate directly to a specific problem that needs solving but rather appears to be an educational or informational passage about trigonometry and the measurement of buildings, followed by a discussion on black holes and the application of Newtonian mechanics. However, I'll attempt to address what seems to be the underlying request for information on how certain principles (like those in physics and mathematics) are applied to real-world problems.
+If we're focusing on the aspect of measuring and structuring buildings safely using trigonometry:
+1. **Understanding Trigonometry**: Trigonometry involves the study of triangles, particularly the relationships between the sides and angles of triangles. This is crucial in architecture and construction for calculating distances, heights, and angles.
+2. **Applications in Building Measurement**:
+   - **Roof Slope Calculation**: The slope of a roof can be determined using trigonometric functions (sine, cosine, tangent) based on the rise over run or the angle of elevation.
+   - **Height Calculations**: For determining the height of buildings or structures without direct measurement, trigonometry is used. By measuring the angle of elevation to the top of the building from a known distance away, one can calculate the height using the tangent function.
+   - **Stairway Design**: The rise and run of stairways are designed with specific ratios to ensure safety and comfort, which can involve trigonometric calculations for precise measurements.
+3. **Video Games and Industrial Machines**:
+   - In video game development, trigonometry is used extensively in game physics (for realistic movements), 3D modeling (to create immersive environments), and collision detection.
+   - For industrial machines and automobiles, trigonometry helps in the design of mechanical parts that involve rotational motion or precise angular measurements.
+Regarding the discussion on black holes and Newtonian mechanics:
+1. **Mass Function and Black Holes**: The mass function \(f(M)\) is a critical tool in astrophysics for determining whether a compact object is likely to be a black hole. If \(f(M) &gt; 3M_{\odot}\) (where \(M_{\odot}\) is the solar mass), it suggests that the object could be a black hole because its mass exceeds the theoretical limit for a neutron star.
+2. **Newtonian Mechanics in Astrophysics**: While general relativity provides a more accurate description of gravity, especially in strong gravitational fields like those near black holes, Newtonian mechanics can still offer useful approximations for many astrophysical phenomena. The calculation of radial velocities and orbital periods, for example, often relies on Newton's laws.
+If there's a specific mathematical problem you'd like help with (e.g., calculating the slope of a roof or determining the mass function for an astrophysical object), please provide more details so I can assist you directly.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -52275,7 +52484,17 @@
       <c r="E30" s="3" t="n"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>It seems like there are two unrelated texts provided. I'll address each separately.
+**Text 1: Black Holes and Trigonometry**
+This text appears to be discussing the detection of black holes using trigonometry and astronomy. The key points are:
+* To determine the mass of a compact object, such as a black hole, astronomers use the mass function (f(M)), which is derived from Kepler's law.
+* The mass function is calculated using the orbital period, radial velocity, and inclination angle of the binary system.
+* If the mass function is greater than 3 solar masses, it is likely that the compact object is a black hole.
+**Text 2: Introduction to Trigonometry**
+This text appears to be an introduction to trigonometry, discussing its applications and basics. The key points are:
+* Trigonometry is used in various fields, such as architecture, engineering, and video game development.
+* The unit circle is a fundamental concept in trigonometry, which helps establish the relationship between sine, cosine, and the coordinates of a point on the circle.
+If you have any specific questions or topics related to these texts that you'd like me to help with, please let me know!</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -52308,7 +52527,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text explores trigonometry concepts, including sine, cosine, and tangent.
+It discusses the unit circle and its relationship to these functions.
+Trigonometry is applied to real-world scenarios, such as building design and measurement.
+The text also touches on color perception and vision, introducing an interactive tool.
+The target audience appears to be students aged 10-14 years old.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -52341,7 +52565,11 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores trigonometry and color perception.
+It discusses sine, cosine, and tangent functions using a unit circle.
+The unit circle shows a direct relationship between sin θ, cos θ, and x, y coordinates.
+Color perception is also explored through digital colors and RGB technology.
+The text aims to educate 10-14 year olds on these concepts.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -52374,7 +52602,11 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers trigonometry, color perception, and vision. 
+It explores sine, cosine, and tangent functions.
+Color mixing and RGB colors are also discussed.
+The role of human vision in updating images is explained.
+Concept mapping is introduced as a tool for organizing information.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -52407,7 +52639,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text explores trigonometry concepts like sine, cosine, and tangent.
+It also touches on human vision and perception, discussing seamless image updates.
+A concept map is introduced as a tool for visualizing thoughts and relationships.
+The physics of color is explained, including how we see objects through light emission and reflection.
+Color originates from light and is perceived by the eye and brain.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -52440,7 +52677,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text explores trigonometry and color physics concepts.
+It discusses sine, cosine, and tangent functions in a circular motion.
+Concept maps are introduced as visual tools for organizing information.
+The physics of color is explained, including human vision and primary colors.
+Primary colors can be combined to generate other colors through additive or subtractive methods.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -52473,7 +52715,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text explores trigonometric functions and color physics.
+It discusses how colors are perceived by the human eye and brain.
+Primary colors and their combinations are explained in detail.
+The visible spectrum and electromagnetic radiation are also covered.
+The text concludes with tips for setting up experiments to test theories related to color and light.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -52506,7 +52753,11 @@
       <c r="E37" s="3" t="n"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers color theory, human vision, and experimentation.
+It discusses how colors are perceived and combined to create new hues.
+Primary colors and their combinations are also explored.
+The role of light and its wavelengths in color perception is explained.
+Experiments with RGB LED lights demonstrate color mixing principles.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -52539,7 +52790,11 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores color theory and vision. 
+It discusses primary colors and their combinations. 
+The human eye can distinguish 10 million colors. 
+Experiments with RGB LED laboratories demonstrate color mixing. 
+Color perception is influenced by wavelength and intensity.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -52572,7 +52827,11 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers experiments and research methods. 
+It discusses trigonometry and RGB LED laboratory experiments. 
+Key tips include designing simple experiments and varying one thing at a time. 
+Conclusions should summarize how results answer the research question. 
+Experiments help learn about something through observation and testing.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -52605,7 +52864,11 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores interactive experiments with trigonometry and RGB LED lights. 
+It discusses observing effects of moving sliders and adjusting values.
+The goal is to learn about cause-and-effect relationships.
+A research question guides the experiment, aiming to draw conclusions.
+The text provides tips for designing effective experiments and writing conclusions.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -52638,7 +52901,11 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores trigonometry and light experiments.
+It discusses observing cosine and tangent values as a dot moves around a circle.
+An RGB LED lab allows adjusting color values to observe effects.
+The text also touches on designing experiments and asking research questions.
+Rainbows and their causes are briefly mentioned.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -52671,7 +52938,11 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers trigonometric functions and light experiments.
+It explores the behavior of COS and TAN theta values in a circle.
+An RGB LED laboratory is introduced for color adjustment experiments.
+Rainbows and their causes are also discussed as a topic of discovery.
+The lesson aims to uncover more about these concepts through interactive experiments.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -52704,7 +52975,12 @@
       <c r="E43" s="3" t="n"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text explores light and color concepts.
+It mentions experiments with TAN values and RGB LED lights.
+The order of adjusting colors can affect results.
+White light is a mixture of colors with different wavelengths.
+The lesson aims to discover more about light and rainbows.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -52737,7 +53013,12 @@
       <c r="E44" s="3" t="n"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+The text discusses an experiment with RGB LED lights and color mixing.
+It references previous lessons about the composition of white light and light waves.
+Students are guided through interactive activities to learn more about colors and wavelengths.
+The topic of rainbows and their causes is introduced for further exploration.
+The lesson aims to help students discover and confirm their understanding of light and colors.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -52770,7 +53051,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+Experimenting with RGB LED and light properties.
+Understanding color mixture and wavelength.
+Exploring prisms and rainbow formation.
+Discovering how colors interact with light.
+Learning about the science of light and color.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -52803,7 +53089,12 @@
       <c r="E46" s="3" t="n"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text reviews concepts about light and color.
+It covers white light as a mixture of colors with different wavelengths.
+Refraction separates colors at different angles, making them visible.
+This phenomenon can create rainbows, which will be explored further.
+The lesson invites interaction and discovery through a program.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -52836,7 +53127,12 @@
       <c r="E47" s="3" t="n"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses the properties of light and color.
+White light is a mixture of colors with different wavelengths.
+Refraction causes each color to bend at a different angle.
+This phenomenon creates colorful events like rainbows.
+The lesson invites exploration and discovery about light and color.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -52869,7 +53165,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses light and its properties.
+It explains how white light refracts into different colors.
+The behavior of light creates colorful events like rainbows.
+An interactive program allows users to explore light refraction.
+The topic is part of a lesson on the properties of light.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -52902,7 +53203,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text explores light refraction and rainbows.
+It describes an interactive program to demonstrate this concept.
+White light is a mixture of colors with different wavelengths.
+Refraction separates these colors, creating a rainbow effect.
+The text also mentions the École polytechnique fédérale de Lausanne (EPFL) university.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -52935,7 +53241,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary of the text:
+The text discusses light refraction and rainbows.
+It explains how white light is refracted at different angles.
+The École polytechnique fédérale de Lausanne (EPFL) is introduced as a research institute.
+The university's history and growth are outlined, from 11 students to 14,000 people.
+The EPFL has become a highly international institution with a strong focus on natural sciences and engineering.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -52968,7 +53279,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers light refraction and rainbows.
+It also discusses the history and development of EPFL (École polytechnique fédérale de Lausanne).
+EPFL has grown rapidly since its inception in 1853.
+The university has a highly international environment with students from over 125 countries.
+EPFL encourages entrepreneurship and has a strong start-up culture among its students.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -53001,7 +53317,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary of the text:
+The text discusses light refraction and rainbows.
+It also covers the history and growth of EPFL, a Swiss university.
+EPFL has become a top international university, attracting students from over 125 countries.
+The university has a selective admission process for international students and a high failure rate for first-year students.
+EPFL is ranked among the world's best universities in various rankings, including QS and Times Higher Education.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -53034,7 +53355,12 @@
       <c r="E53" s="3" t="n"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses the properties of light and its refraction, creating rainbows. 
+It also covers the history and growth of EPFL, a Swiss university.
+EPFL has become highly international, attracting students and researchers worldwide.
+The university has a selective admission process for international students.
+EPFL ranks high in various global university rankings, particularly in engineering and technology.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -53067,7 +53393,12 @@
       <c r="E54" s="3" t="n"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+EPFL is a top-ranked university with a strong focus on engineering and technology.
+The university has grown rapidly since its founding in 1969, with over 14,000 students and staff from 125 countries.
+Admission to EPFL is selective for international students, but not for Swiss residents who hold a maturité certificate.
+EPFL ranks highly in international university rankings, including QS World University Rankings and Times Higher Education.
+The university is known for its strong scientific impact, international outlook, and faculty-to-student ratio.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -53100,7 +53431,15 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text appears to be a humorous article about giving cats an annual performance review. The author provides tongue-in-cheek guidelines on how to evaluate a cat's performance, including setting standards based on age and breed, focusing on impact, and providing specific feedback.
+Some of the key points from the article include:
+1. Evaluating a cat's performance against a standard that takes into account their age and breed.
+2. Using the situation-behavior-impact (SBI) model to provide specific and actionable feedback.
+3. Creating a performance improvement plan (PIP) when a cat is not meeting expectations.
+4. Providing regular individual feedback and acknowledging positive behaviors.
+5. Being aware of one's own role in a cat's performance, such as providing adequate space and toys.
+The article is written in a lighthearted and satirical tone, with the author using humorous examples and anecdotes to illustrate their points. It is not meant to be taken seriously, but rather as an entertaining and playful take on the idea of giving cats a performance review.
+In contrast, the first part of the text appears to be about a university or academic institution, specifically École polytechnique fédérale de Lausanne (EPFL), and its admission requirements and procedures. It seems unrelated to the rest of the text, which is about cat performance reviews.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -53137,7 +53476,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses university rankings, specifically EPFL's rankings in Engineering and Technology.
+EPFL is ranked highly in various categories, including faculty to student ratio and scientific impact.
+The university also ranks well in international outlook and citation index.
+In contrast, the text also includes a satirical piece about giving cats their annual performance review.
+The two topics seem unrelated, with the first discussing academic rankings and the second being a humorous take on cat ownership.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -53174,7 +53518,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The article humorously discusses giving annual performance reviews to cats.
+It outlines guidelines for evaluating cat performance, including setting standards and goals.
+Feedback should be specific, actionable, and focused on impact.
+A performance improvement plan may be necessary for underperforming cats.
+The article uses satire to poke fun at management techniques and cat ownership.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -53207,7 +53556,11 @@
       <c r="E58" s="3" t="n"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The article satirically discusses giving annual performance reviews to cats. 
+It outlines guidelines for evaluating a cat's performance, including setting standards and focusing on impact.
+The article uses humor to convey the importance of constructive feedback and appreciation.
+Regular individual feedback sessions are recommended to address negative behaviors and praise positive ones.
+The tone is lighthearted and comedic, using satire to poke fun at management and leadership techniques.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -53244,7 +53597,11 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses functional modeling for estimating power.
+It provides a model to evaluate and estimate power usage.
+The example given is an electric car with a battery and motor.
+The goal is to assess if the model is useful for estimation.
+Functional modeling helps understand how systems work.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -53277,7 +53634,11 @@
       <c r="E60" s="3" t="n"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses functional modeling for estimating power.
+It provides a model to evaluate and estimate power usage.
+The topic of electric cars is introduced as an example.
+A basic explanation of how an electric car works is given.
+Functional modeling is used to understand and reflect on the process.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -53314,7 +53675,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+Electric cars run on batteries that power electric motors.
+They have no tailpipe or gas tank, reducing emissions and maintenance needs.
+The motor and controller work together to regulate energy use.
+Regenerative braking recharges the battery using the car's momentum.
+Overall, electric cars offer an efficient and environmentally friendly alternative.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -53351,7 +53717,12 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+The text describes how an electric car works, highlighting its key components. 
+It explains the role of the battery and electric motor in powering the vehicle.
+The electric car's structure is similar to fossil fuel-powered cars but lacks a tailpipe and gas tank.
+Regenerative braking allows the car to recharge its battery using the motor's momentum.
+Overall, the text provides an overview of electric car technology and its advantages.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -53388,7 +53759,11 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Electric cars have a similar structure to fossil fuel-powered cars but lack a tailpipe and gas tank. 
+They are powered by an electric motor and battery, which supplies energy for acceleration. 
+The electric motor requires no oil or tune-ups and produces no emissions. 
+Regenerative braking is used to recharge the battery when the brakes are applied. 
+Overall, electric cars have several advantages over traditional fossil fuel-powered vehicles.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -53425,7 +53800,8 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+Electric cars have a similar structure to fossil fuel-powered cars but lack a tailpipe and gas tank. They are powered by an electric motor and battery, which supplies energy for acceleration. The controller regulates power to prevent the motor from burning out. Regenerative braking recharges the battery using the motor's momentum when brakes are applied. Electric cars have several advantages, including no oil or tune-ups required and reduced emissions.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -53462,7 +53838,11 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Electric cars have a similar structure to fossil fuel-powered cars but lack a tailpipe and gas tank. 
+They are powered by an electric motor and battery, which provides acceleration and energy. 
+The electric motor requires no oil or tune-ups and produces no emissions. 
+Regenerative braking allows the car to recharge its battery using the motor's momentum. 
+Overall, electric cars offer a sustainable and efficient alternative to traditional vehicles.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -53495,7 +53875,12 @@
       <c r="E66" s="3" t="n"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+Electric cars have a similar structure to fossil fuel-powered cars.
+They are powered by an electric motor and battery, with no tailpipe or gas tank.
+The electric motor provides acceleration and requires no oil or tune-ups.
+Regenerative braking allows the car to recharge its battery using momentum.
+This makes electric vehicles efficient and environmentally friendly.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -53528,7 +53913,11 @@
       <c r="E67" s="3" t="n"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Electric cars have a similar structure to fossil fuel-powered cars but lack a tailpipe and gas tank. 
+They are powered by an electric motor and battery, which supplies energy for movement.
+The controller regulates power to prevent the motor from burning out.
+Regenerative braking recharges the battery using the motor's momentum when brakes are applied.
+Electric cars offer advantages like reduced emissions and lower maintenance needs.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -53561,7 +53950,11 @@
       <c r="E68" s="3" t="n"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Electric cars have a similar structure to fossil fuel-powered cars but with an electric motor and battery. 
+The electric motor requires no oil or tune-ups and produces no emissions. 
+The battery powers the motor and electronic devices, providing acceleration and energy efficiency. 
+Regenerative braking allows the car to recharge its battery using the motor's momentum. 
+Overall, electric cars offer a sustainable and efficient alternative to traditional vehicles.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -53594,7 +53987,12 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses electric cars and their components. 
+Electric cars have an electric motor, controller, and battery as the power source.
+Regenerative braking is used to recharge the battery when the car brakes.
+The text also touches on quantitative modeling and evaluation of electric car parameters.
+It relates to the topic of particulate nature of matter and rate of diffusion.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -53627,7 +54025,12 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses electric cars and their components. 
+Electric cars have an electric motor, controller, and battery as the power source. 
+Regenerative braking allows the car to recharge its battery using momentum. 
+The overall structure of an electric car is similar to a fossil fuel-powered car. 
+The text also mentions diffusion and factors affecting its rate.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -53660,7 +54063,11 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses the topic of diffusion in the context of particulate matter.
+It explores factors affecting the rate of diffusion, including temperature.
+The objective is to determine these factors and understand their impact.
+The text also touches on estimation problems related to calculating power.
+Diffusion and its relationship with temperature are key themes.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -53693,7 +54100,11 @@
       <c r="E72" s="3" t="n"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses lab experiments and predictions.
+It covers the topic of particulate nature of matter, specifically rate of diffusion.
+The objective is to determine factors affecting rate of diffusion.
+Temperature's effect on rate of diffusion is a key point of inquiry.
+Lab work involves predicting outcomes and testing hypotheses.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -53726,7 +54137,11 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers lab experimentation and prediction.
+It involves understanding diffusion and its factors.
+Temperature and molecular mass affect the rate of diffusion.
+An experiment is outlined with steps to regulate temperature and molecular mass.
+The goal is to test predictions and observe molecular interactions.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -53759,7 +54174,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses experimentation and prediction in a lab setting.
+It also explores the effect of temperature on the rate of diffusion.
+Additionally, it touches on the process of photosynthesis in plants.
+Photosynthesis is crucial for plant survival, using light energy to produce food.
+The experiment involves regulating temperature and molecular mass to observe molecule interactions.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -53792,7 +54212,11 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers experiment planning and execution.
+It involves predicting outcomes and testing hypotheses.
+Photosynthesis is introduced as a process by which plants produce food from light energy.
+Plants require light to survive and release oxygen as a byproduct.
+The experiment will explore how light affects photosynthesis in aquarium plants.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -53825,7 +54249,11 @@
       <c r="E76" s="3" t="n"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses photosynthesis in plants, specifically in aquarium plants.
+It explores how light intensity affects photosynthesis.
+An experiment is outlined to investigate this relationship.
+Plants use light energy to produce food through photosynthesis, releasing oxygen as a byproduct.
+The process occurs in the green parts of plants and is essential for their survival.</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -53858,7 +54286,12 @@
       <c r="E77" s="3" t="n"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses photosynthesis in aquarium plants.
+It explores how light intensity affects photosynthesis.
+The experiment also examines seasonal effects on photosynthesis.
+Plants use light energy to produce food through photosynthesis.
+The process releases oxygen as a byproduct.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -53891,7 +54324,12 @@
       <c r="E78" s="3" t="n"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+Photosynthesis in plants depends on light intensity and season.
+Plants use light energy to make food through photosynthesis.
+This process occurs in green parts of plants and releases oxygen.
+Aquarium plants' photosynthesis will be explored in relation to light and season.
+The experiment aims to understand how these factors affect plant growth.</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -53924,7 +54362,12 @@
       <c r="E79" s="3" t="n"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses photosynthesis in plants, a process using light energy to produce food.
+Plants require light, carbon dioxide, water, nutrients, and minerals for photosynthesis.
+Photosynthesis occurs in green parts of plants and releases oxygen as a byproduct.
+The text also touches on collaborative work and experimental procedures.
+Aquarium plants' photosynthesis is affected by light and the season of the year.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -53957,7 +54400,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses plant survival and food production through photosynthesis.
+Photosynthesis uses light energy, carbon dioxide, water, and nutrients to produce oxygen.
+It occurs in green parts of plants and is essential for their survival.
+The text also touches on collaborative work and problem-solving strategies.
+Aquarium plants' photosynthesis is explored in relation to seasonal changes.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -53990,7 +54438,12 @@
       <c r="E81" s="3" t="n"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses collaborative work challenges.
+It also explores plant photosynthesis and its importance.
+Plants produce oxygen through photosynthesis using light energy.
+The process occurs in green parts of plants.
+Investigations on light and season effects on photosynthesis are also mentioned.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -54023,7 +54476,11 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers collaborative work challenges and improvements.
+It also explores plant management for ammonia production.
+Photosynthesis in aquarium plants is another topic discussed.
+The Haber process for synthesizing ammonia is introduced.
+Managing variables to optimize production is a key theme.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -54056,7 +54513,12 @@
       <c r="E83" s="3" t="n"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+The text discusses a collaborative task involving ammonia production.
+It requires managing a plant to produce as much ammonia as possible.
+The Haber process is used to synthesize ammonia from nitrogen and hydrogen.
+Independent variables can be adjusted to analyze results and optimize production.
+The goal is to produce the maximum amount of NH3 at the least cost.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -54089,7 +54551,8 @@
       <c r="E84" s="3" t="n"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text covers various scientific topics, including plant management and ammonia production. It also touches on biology, specifically the mammalian eye and photosynthesis. Additionally, it mentions transcription and translation concepts. The Haber process for synthesizing ammonia is discussed in detail. Overall, the text explores different scientific investigations and experiments.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -54122,7 +54585,12 @@
       <c r="E85" s="3" t="n"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers various scientific topics, including the mammalian eye and its parts.
+It also explores photosynthesis in aquarium plants and its relation to light and season.
+Additionally, transcription and translation concepts are introduced through a YouTube video.
+The Haber process for synthesizing ammonia is discussed with a focus on optimization.
+These topics aim to provide interactive learning experiences through labs and simulations.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -54155,7 +54623,11 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers the structure and function of the mammalian eye. 
+It explains the role of parts like cornea, lens, and retina in sight perception.
+The text also touches on a lab investigation about light reflection and iris control.
+Additionally, it mentions the Haber process for ammonia synthesis.
+The overall theme is biology and chemistry concepts.</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -54188,7 +54660,11 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers the structure and function of the mammalian eye. 
+It explains how different parts work together to enable sight. 
+The eye is compared to a camera with similar components. 
+Light perception and conversion to electrochemical impulses are key functions. 
+The text also touches on the Haber process for ammonia synthesis.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -54221,7 +54697,11 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The mammalian eye is a sensory organ with parts adapted for sight.
+It has photo receptors that perceive light as a stimulus.
+The eye's components work like a camera to provide clear vision.
+The cornea, lens, retina, and iris all play vital roles in focusing light.
+The human eye converts light into electrochemical impulses, allowing us to see.</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -54254,7 +54734,11 @@
       <c r="E89" s="3" t="n"/>
       <c r="F89" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The mammalian eye is a sensory organ with parts adapted for perception of light. 
+It has cornea, lens, retina, and iris that work together for clear vision. 
+The eye functions like a camera, focusing light onto the retina. 
+Rod and cone cells in the retina convert light to electrochemical impulses. 
+The human eye accommodates changing lighting conditions and focuses light rays for sharp vision.</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -54287,7 +54771,11 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The mammalian eye has various parts adapted for perception of sight.
+It includes the cornea, lens, retina, and iris, each playing a vital role.
+The eye works similarly to a camera, with each part contributing to clear vision.
+The retina converts light into electrical impulses sent to the brain.
+The human eye accommodates changing lighting conditions and focuses light rays.</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -54320,7 +54808,11 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The mammalian eye is a sensory organ with photo receptors.
+It has various parts, including cornea, lens, and retina, adapted to their functions.
+The retina converts light rays into electrical impulses sent to the brain.
+The eye accommodates changing lighting conditions and focuses light rays from varying distances.
+The proper functioning of all components allows for image perception.</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -54353,7 +54845,12 @@
       <c r="E92" s="3" t="n"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The mammalian eye has multiple parts that work together for sight perception.
+Key components include the cornea, lens, retina, and iris, which control light entry.
+The retina converts light rays into electrical impulses sent to the brain.
+The macula enables sharp vision, while the peripheral retina handles peripheral vision.
+Proper functioning of these components allows the eye to focus and perceive images.</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -54386,7 +54883,11 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers the structure of the mammalian eye and its parts. 
+It mentions the cornea, lens, retina, and iris and their roles. 
+The text also briefly touches on DNA and nucleotides. 
+It describes the components of a nucleotide, including nitrogenous base and phosphate group. 
+The topic seems to be a transition between biology lessons on vision and molecular biology.</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -54419,7 +54920,12 @@
       <c r="E94" s="3" t="n"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text reviews DNA structure and nucleotides.
+It reminds readers of key components: nitrogenous bases, sugar, and phosphate groups.
+Concentrated and dilute solutions are also defined.
+The lesson is entering its second phase, Conceptualization.
+Readers are encouraged to recall prior knowledge before moving forward.</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -54452,7 +54958,11 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text reviews DNA structure and nucleotides.
+It covers the components of nucleotides, including nitrogenous bases.
+The concept of dilute solutions is also mentioned briefly.
+The text prepares for a lesson phase focused on conceptualization.
+Key concepts include DNA, nucleotides, and proteins.</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -54485,7 +54995,11 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text reviews DNA structure and nucleotides.
+It covers nitrogenous bases, sugar, and phosphate groups.
+The lesson is in its second phase, Conceptualization.
+The goal is to reinforce prior knowledge before moving forward.
+Key concepts include DNA, nucleotides, and amino acids.</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -54518,7 +55032,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text reviews DNA structure and nucleotides.
+It also covers proteins and amino acids.
+Genetic information directs protein synthesis in ribosomes.
+The genetic code consists of codons, with three bases per amino acid.
+A gene encodes a specific protein through its sequence of bases.</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -54551,7 +55070,12 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The text reviews DNA structure and nucleotides.
+It discusses the concept of genetic information directing protein synthesis.
+The sequence of bases in DNA encodes a protein like a recipe book.
+A gene is a sequence of bases encoding a particular protein.
+The laboratory simulation demonstrates transcription with base pairing rules.</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -54584,7 +55108,12 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text reviews DNA structure and nucleotides.
+It discusses genetic information directing protein synthesis in cells.
+The sequence of bases in DNA codes for protein creation.
+A gene encodes a specific protein through codons and base pairing.
+The process involves transcription, mRNA formation, and translation to ribosomes.</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -54617,7 +55146,12 @@
       <c r="E100" s="3" t="n"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The structure of DNA and nucleotides is reviewed.
+Genetic information directs protein synthesis in cell ribosomes.
+The sequence of bases in DNA codes for protein creation.
+A gene is a sequence of bases encoding a particular protein.
+The process involves transcription and translation to create proteins.</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -54650,7 +55184,12 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text reviews DNA structure and nucleotides.
+It discusses transcription and translation processes in cells.
+mRNA molecules carry genetic information from the nucleus to the cytoplasm.
+Translation occurs at ribosomes, where tRNA brings amino acids to form proteins.
+The process results in protein synthesis with specific amino acid sequences.</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -54683,7 +55222,11 @@
       <c r="E102" s="3" t="n"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers scientific concepts, including DNA and RNA.
+It references a historical story about Archimedes and a golden crown.
+The laboratory section explores DNA transcription and translation.
+The process of protein synthesis is described, involving mRNA and tRNA molecules.
+Key biological concepts are introduced, preparing students for the next course phase.</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -54716,7 +55259,12 @@
       <c r="E103" s="3" t="n"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text covers various topics including Archimedes' discovery of fraud in a golden crown.
+It also features a personal story of buying a dream car, an AM General Hummer H1.
+Additionally, the text discusses DNA transcription and translation processes.
+It includes interactive lab simulations for learning about base pairing rules and protein synthesis.
+The topics appear to be unrelated, covering history, cars, and molecular biology.</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -54749,7 +55297,13 @@
       <c r="E104" s="3" t="n"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text covers three unrelated topics: 
+Archimedes and Vitruvius' story about a golden crown.
+A car enthusiast's video about buying and testing an AM General Hummer H1.
+A biology lesson on DNA transcription and translation, including RNA and protein synthesis. 
+These topics are distinct and separate from one another.
+The text includes various links and disclaimers related to the car video.</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -54782,7 +55336,11 @@
       <c r="E105" s="3" t="n"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers various topics including buying a dream car, off-roading, and car-related content. 
+It also mentions robotic arm geometry and DNA transcription. 
+Additionally, it touches on protein synthesis and translation. 
+The content is from different YouTube videos and sources. 
+Overall, it's a mix of automotive and scientific topics.</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -54815,7 +55373,12 @@
       <c r="E106" s="3" t="n"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers robotic arm geometry and types. 
+It explains rectangular, cylindrical, spherical, and jointed spherical arms.
+Additionally, it touches on DNA transcription and translation processes.
+mRNA molecules carry genetic information from the nucleus to the cytoplasm.
+The process involves tRNA and rRNA molecules in protein synthesis.</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -54848,7 +55411,11 @@
       <c r="E107" s="3" t="n"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers robotic arm geometry and DNA transcription. 
+It explains four types of robotic arms and their movements.
+It also discusses DNA transcription and translation processes.
+The role of RNA molecules, including tRNA and rRNA, is highlighted.
+Key concepts in biology and engineering technology are explored.</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -54881,7 +55448,12 @@
       <c r="E108" s="3" t="n"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text covers various unrelated topics. 
+It touches on robotics, racism, and molecular biology.
+Racism is discussed from a social learning perspective.
+Molecular biology concepts, such as DNA transcription and translation, are also explored.
+These topics seem to be unrelated and lack a cohesive theme.</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -54914,7 +55486,11 @@
       <c r="E109" s="3" t="n"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers racism and its effects on society. 
+It examines the root causes from a social learning perspective.
+Additionally, it touches on DNA transcription and translation.
+The process of creating mRNA molecules is described.
+Racism and molecular biology are the two main topics discussed.</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -54947,7 +55523,12 @@
       <c r="E110" s="3" t="n"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+Racism is prejudice based on the belief of racial superiority.
+It has a profound impact on humanity, degrading our future.
+The root causes and effects of racism will be examined from a social learning perspective.
+The text also touches on DNA transcription and translation in a virtual lab setting.
+Understanding these concepts will lead to further discussion and exploration in the course.</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -54980,7 +55561,12 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses racism and its impact on society.
+It explores the root causes of racism from a social learning perspective.
+However, the text also abruptly changes topic to discuss molecular biology and genetics.
+Additionally, it covers the rectilinear propagation of light and its properties.
+Overall, the text touches on three unrelated topics: racism, molecular biology, and physics.</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -55013,7 +55599,12 @@
       <c r="E112" s="3" t="n"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers two main topics: racism and molecular biology.
+It discusses protein synthesis and translation of DNA.
+RNA molecules, including tRNA and rRNA, play a crucial role in this process.
+The text also explores the property of rectilinear propagation of light.
+Light travels in a straight line, forming shadows and day-night cycles.</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -55046,7 +55637,13 @@
       <c r="E113" s="3" t="n"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers two main topics: 
+Racism and molecular biology experiments.
+It explains protein synthesis and translation of DNA.
+Transfer RNA (tRNA) and ribosomal RNA (rRNA) are discussed.
+The second part shifts to physics, discussing light propagation.
+Rectilinear propagation of light is demonstrated through an experiment.</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -55079,7 +55676,12 @@
       <c r="E114" s="3" t="n"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text covers lab experiments and scientific concepts.
+It discusses DNA translation and protein synthesis.
+The role of mRNA, tRNA, and rRNA molecules is explained.
+The rectilinear propagation of light is demonstrated through experiments.
+Light travels in a straight line, forming shadows and day-night cycles.</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -55112,7 +55714,12 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers lab experiments and scientific concepts.
+It introduces the Experiment Lab and Bending Light Lab for hands-on learning.
+DNA translation, tRNA, and rRNA are explained in the context of protein formation.
+The rectilinear propagation of light is demonstrated through experiments and examples.
+The topics range from biology to physics and mathematics, including quadratic equations.</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -55145,7 +55752,12 @@
       <c r="E116" s="3" t="n"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers lab experiments and equipment usage.
+It discusses translation of DNA and RNA molecules' roles.
+Rectilinear propagation of light is also explored with demonstrations.
+The formation of shadows, eclipses, and day/night cycles are explained.
+Quadratic equations and algebra topics are mentioned as additional learning material.</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -55178,7 +55790,12 @@
       <c r="E117" s="3" t="n"/>
       <c r="F117" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers various science topics, including light propagation and genetics.
+It discusses rectilinear propagation of light and its consequences.
+The translation of DNA into amino acids is also explained.
+Quadratic equations and algebra are mentioned as additional topics.
+These subjects are covered through labs, videos, and demonstrations.</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -55211,7 +55828,13 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text covers two main topics: 
+Light propagation and quadratic equations.
+It discusses rectilinear propagation of light and its examples.
+Quadratic equations are also introduced with a focus on graphical solutions.
+The quadratic formula is mentioned as a tool for solving equations.
+Key concepts include light traveling in straight lines and algebraic problem-solving.</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -55244,7 +55867,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text discusses solving quadratic equations.
+It mentions using the quadratic formula and graphical methods.
+The quadratic formula is used to find values of x.
+Resources are provided for further learning, including videos and websites.
+Quadratic equations can be solved when y=0 and a, b, c are known.</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -55277,7 +55905,11 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses solving quadratic equations.
+It mentions using graphical methods to find solutions.
+A website, MathMeeting.com, offers free algebra videos.
+Quadratic equations can be solved when y=0 and a, b, c are known.
+Graphical and formula methods yield the same results for x.</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -55310,7 +55942,11 @@
       <c r="E121" s="3" t="n"/>
       <c r="F121" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses solving quadratic equations using graphs.
+It provides examples and resources, including free videos.
+The graphical method involves setting y=0 to find x values.
+This approach yields the same results as other methods.
+Quadratic equations can be solved graphically with known coefficients a, b, and c.</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -55343,7 +55979,11 @@
       <c r="E122" s="3" t="n"/>
       <c r="F122" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers solving quadratic equations using graphs.
+It discusses two methods for solving quadratic equations.
+Both methods yield the same results for x values.
+Leadership qualities and self-motivation are also briefly mentioned.
+Quadratic equations can be solved graphically with known coefficients.</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -55376,7 +56016,11 @@
       <c r="E123" s="3" t="n"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses achieving success in life through leadership qualities. 
+It touches on solving quadratic equations using two methods. 
+Both methods yield the same results for x when y=0 and a, b, c are known.
+Leadership is analyzed as a key factor in goal achievement.
+Success requires endurance, self-motivation, and strong character traits.</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -55409,7 +56053,12 @@
       <c r="E124" s="3" t="n"/>
       <c r="F124" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses finding purpose in life and achieving success.
+It highlights the importance of leadership qualities, endurance, and self-motivation.
+The topic of leadership and its variations is introduced for analysis.
+A quote suggests that leadership is about action and example, not just position or title.
+The text also briefly mentions solving quadratic equations, but this seems unrelated to the main theme.</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -55442,7 +56091,11 @@
       <c r="E125" s="3" t="n"/>
       <c r="F125" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses leadership and its true meaning. 
+It emphasizes that leadership is about action, not title. 
+The conversation then shifts to quadratic equations. 
+Graphical and formula methods can solve these equations. 
+Both methods yield the same results for x.</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -55475,7 +56128,12 @@
       <c r="E126" s="3" t="n"/>
       <c r="F126" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text explores leadership and its true meaning.
+It discusses what leadership in Utopia would look like.
+Lars Sudmann shares strategies on self-leadership to develop into a "Utopia leader".
+The talk highlights personal journeys of great leaders and lessons from the golden age of leadership.
+Leadership is about action and example, not just position or title.</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -55508,7 +56166,12 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The concept of leadership is discussed, emphasizing action and example.
+A TEDxUtopia talk explores what leadership in Utopia would look like.
+Lars Sudmann shares strategies for self-leadership development.
+He draws from personal journeys of great leaders and historical lessons.
+The goal is to develop into a "Utopia leader" with effective leadership skills.</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -55541,7 +56204,12 @@
       <c r="E128" s="3" t="n"/>
       <c r="F128" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses leadership in Utopia and strategies for self-leadership.
+It references a TEDx talk by Lars Sudmann on overcoming the "leadership formula of doom".
+Practical tasks are also mentioned, including testing pH levels of coffee and soap.
+Additionally, mathematical concepts, such as solving for x, are touched upon.
+The text covers various topics, including leadership, chemistry, and problem-solving.</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -55574,7 +56242,12 @@
       <c r="E129" s="3" t="n"/>
       <c r="F129" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses leadership in Utopia and strategies for self-leadership.
+It explores the "leadership formula of doom" and how great leaders overcome it.
+Additionally, the text touches on chemistry concepts, including pH levels and acid-base reactions.
+It also mentions procedures for testing pH levels and predicting color changes.
+Overall, the text covers leadership development and basic chemistry principles.</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -55607,7 +56280,12 @@
       <c r="E130" s="3" t="n"/>
       <c r="F130" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers experiments with pH levels of coffee and soap.
+It explores how volume changes affect acidity and basicity.
+Acids have a pH of 1-6, while bases have a pH of 8-14.
+A brief mention of the Digital Divide is made, but not elaborated on.
+The text also touches on solving equations and predicting color changes in solutions.</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -55640,7 +56318,12 @@
       <c r="E131" s="3" t="n"/>
       <c r="F131" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text covers multiple topics, including chemistry and digital divide.
+Acids and bases react to form neutral solutions with specific pH levels.
+The digital divide lesson aims to educate students on its meaning and effects.
+It also explores old and new economies and their features.
+Chemistry and math concepts are also briefly mentioned.</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -55673,7 +56356,11 @@
       <c r="E132" s="3" t="n"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The lesson covers the concept of Digital Divide.
+It aims to explain the meaning and features of old and new economies.
+The impact of Digital Divide on people's lives is also discussed.
+A video is provided for better understanding.
+The topic focuses on digital inequality and its effects.</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -55706,7 +56393,12 @@
       <c r="E133" s="3" t="n"/>
       <c r="F133" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The digital divide refers to unequal access to information technology.
+It affects people's lives and can be classified by gender, income, and location.
+Global digital divide occurs between countries with differing technological access.
+The concept describes the gap between those with and without effective access to ICT.
+Understanding the digital divide is crucial for explaining its impact on society.</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -55739,7 +56431,11 @@
       <c r="E134" s="3" t="n"/>
       <c r="F134" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to unequal access to ICT.
+It affects people based on gender, income, and location.
+Global digital divide occurs between countries.
+This gap limits access to information and technology.
+It's a societal issue with significant implications.</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -55772,7 +56468,11 @@
       <c r="E135" s="3" t="n"/>
       <c r="F135" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to unequal access to technology.
+It affects people based on gender, income, and location.
+Global digital divide exists between countries with varying technological access.
+This gap separates those with internet access from those without.
+The digital divide highlights societal disparities in ICT access.</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -55805,7 +56505,11 @@
       <c r="E136" s="3" t="n"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to the gap in internet access between demographics and regions.
+Half of the world's population remains offline, with Africa having the highest percentage without connection.
+The digital divide affects not only access but also quality of infrastructure and digital literacy.
+Digital technologies can boost economic growth and education, but benefits are unevenly distributed.
+Closing the gap in internet access is critical for global participation in the digital economy.</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -55838,7 +56542,11 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to the gap between those with internet access and those without.
+Half of the world's population remains offline, with Africa having 88% without connection.
+The divide also encompasses disparities in digital infrastructure and skills.
+Digital technologies bring numerous benefits, but unevenly distributed due to limited connectivity.
+Closing the internet access gap is critical for global participation in the digital economy.</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -55871,7 +56579,11 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to the gap between those with internet access and those without. 
+Half of the world's population remains offline, with Africa having 88% without connection.
+The divide also includes discrepancies in digital infrastructure and skills.
+Closing the gap is crucial for global participation in the digital economy.
+Innovative solutions are needed to deploy technology sustainably and affordably.</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -55904,7 +56616,11 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to the gap between those with access to modern technology and those without. 
+Half of the world's population lacks internet access, with Africa having the highest percentage. 
+The digital divide encompasses not only access but also quality and skills. 
+Digital technologies can boost economic growth and education, but benefits are unevenly distributed. 
+Closing the gap in internet access is critical for global prosperity.</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -55937,7 +56653,11 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to the gap between those with internet access and those without. 
+Half of the world's population remains offline, with Africa having the highest percentage.
+The digital divide affects not only access but also quality of infrastructure and digital literacy.
+Closing this gap is critical for global prosperity and economic growth.
+Innovative solutions are needed to address the digital divide and promote equitable use of technology.</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -55970,7 +56690,11 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to the gap in internet access between demographics and regions. 
+Half of the world's population remains offline, with Africa having the highest percentage without connection. 
+The digital divide encompasses not only access but also quality of infrastructure and digital literacy. 
+Digital technologies can bring economic growth and opportunities, but benefits are unevenly distributed. 
+Closing the gap in internet access is critical for global prosperity and participation in the digital economy.</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -56007,7 +56731,11 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The digital divide refers to unequal internet access globally.
+Half of the world's population remains offline, with Africa at 88% disconnected.
+The gap affects not only access but also quality and skills.
+Digital technologies can boost economies and education, but benefits are unevenly distributed.
+Closing the gap is critical for global prosperity and digital equality.</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -56040,7 +56768,12 @@
       <c r="E143" s="3" t="n"/>
       <c r="F143" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The world faces a digital divide, with half the population offline.
+Asia has the most people without internet, while Africa has the highest percentage.
+Male internet users outnumber females in every region.
+Digital technologies can boost economies and improve education, but benefits are unevenly distributed.
+Closing the gap in internet access is critical for global prosperity.</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -56073,7 +56806,8 @@
       <c r="E144" s="3" t="n"/>
       <c r="F144" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text covers various topics, including three-dimensional geometry and sexual selection in guppies. It mentions objectives of 3D geometry and variables in a virtual laboratory. The text also references a research article on natural selection in guppies. Additionally, it lists geometrical properties and angles between lines and planes. Key concepts include skew lines and projection of a line onto a plane.</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -56106,7 +56840,12 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The text covers objectives of Three Dimensional Geometry.
+It includes topics such as geometrical properties and angles between lines and planes.
+Natural selection and UV radiation are also mentioned in separate contexts.
+The text references a research article on natural selection in guppies.
+It concludes with an invitation to collaborate on a project measuring UV levels.</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -56139,7 +56878,12 @@
       <c r="E146" s="3" t="n"/>
       <c r="F146" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses ultraviolet radiation and its effects on humans.
+It touches on the importance of protection from UV radiation.
+A project is mentioned where students measure UV levels in their town.
+The project also studies awareness of UV radiation among family members.
+Students can collaborate globally to compare their results.</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -56172,7 +56916,12 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses ultraviolet radiation and its effects on humans.
+It highlights the importance of protection from UV radiation.
+A project is mentioned where students measure UV levels and awareness in their town.
+The project uses UV light sensitive beads and a standardized UV scale.
+Students can compare results with others worldwide using online resources.</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -56205,7 +56954,12 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses the effects of ultraviolet radiation on the skin.
+It highlights the importance of protection from UV radiation worldwide.
+A project is introduced where students measure UV levels and study awareness in their community.
+The project uses UV-sensitive beads and a standardized UV scale for comparison.
+Students can experiment with different sunscreens to test their effectiveness in blocking UV radiation.</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -56238,7 +56992,12 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses ultraviolet radiation and its effects on the skin.
+It introduces the UV Index, a standardized scale measuring UV radiation levels worldwide.
+An experiment is proposed to test different methods of protecting skin from UV radiation.
+Materials needed include UV sensitive beads, sunscreen, and a UV level scale.
+The goal is to determine effective ways to block UV radiation and protect the skin.</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -56271,7 +57030,12 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses ultraviolet radiation and its effects on skin.
+An experiment is proposed to test methods of protection from UV radiation.
+Materials needed include UV sensitive beads, sunscreen, and a UV level scale.
+The goal is to evaluate effective and non-effective ways to block UV radiation.
+The activity aims to raise awareness about UV rays and their dangers.</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -56304,7 +57068,12 @@
       <c r="E151" s="3" t="n"/>
       <c r="F151" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses ultraviolet radiation and its effects on the skin.
+It encourages readers to develop an hypothesis on how to protect themselves from UV radiation.
+An experiment is proposed to test different methods of protection, including sunscreen with various protective factors.
+The goal is to determine which methods are effective in blocking UV radiation.
+The activity aims to educate readers about UV rays and promote awareness of skin protection.</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -56337,7 +57106,12 @@
       <c r="E152" s="3" t="n"/>
       <c r="F152" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses ultraviolet radiation and its effects on skin.
+It encourages readers to develop an hypothesis on how to protect themselves from UV radiation.
+An experiment is proposed to test different methods of blocking UV radiation.
+Materials such as UV sensitive beads, sunscreen, and a UV level scale are needed for the experiment.
+The goal is to learn about effective ways to protect skin against UV damage.</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -56370,7 +57144,12 @@
       <c r="E153" s="3" t="n"/>
       <c r="F153" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers an experiment to test sunscreen protection against UV radiation.
+Students develop a hypothesis and test various protective factors.
+Materials include UV sensitive beads, sunscreen, and a UV level scale.
+The goal is to evaluate effective ways to block UV radiation.
+The activity teaches about UV benefits, dangers, and skin protection methods.</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -56403,7 +57182,12 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses an interactive science activity involving acids, bases, and UV rays.
+Students develop hypotheses and conduct experiments to learn about these concepts.
+They evaluate their community's awareness of UV risks and explore protective measures.
+The activity involves using an app to investigate substances and their acidity or basicity.
+It aims to educate students about the benefits and dangers of UV rays.</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -56436,7 +57220,12 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text covers science activities and experiments. 
+It involves exploring acids and bases, UV rays, and their effects.
+Students develop hypotheses and investigate substances using an app.
+They learn about protecting skin from UV damage and chemical reactions.
+The goal is to educate students about science concepts in a interactive way.</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -56469,7 +57258,11 @@
       <c r="E156" s="3" t="n"/>
       <c r="F156" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers acids and bases, including their dangers.
+It mentions a reaction between hydrochloric acid and calcium carbonate.
+The topic of UV rays and skin protection is also introduced.
+An interactive activity is suggested to investigate acidic and basic substances.
+Chemical reactions and safety are key themes in the text.</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -56502,7 +57295,12 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers acids and bases, including their reactions.
+Marble reacts with hydrochloric acid due to its calcium carbonate composition.
+A simple electrical circuit consists of a wire, battery, and bulb connected in series.
+Conductive parts must connect in a closed circular arrangement for the circuit to work.
+The battery creates voltage, forcing electrons to flow from negative to positive.</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -56535,7 +57333,12 @@
       <c r="E158" s="3" t="n"/>
       <c r="F158" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers acids and bases, including their reaction with calcium carbonate.
+It also discusses electrical circuits and their components, such as wires and batteries.
+A simple electrical circuit requires a closed circular arrangement of conductive parts.
+The battery creates a potential difference, or voltage, that forces electrons to flow.
+Electrical circuits and chemical reactions are the main topics explored in the text.</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -56568,7 +57371,12 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text covers acids and bases, electrical circuits, and scientific hypotheses.
+It explains how calcium carbonate reacts with hydrochloric acid.
+A simple electrical circuit requires a wire, battery, and bulb connected in series.
+Conductive parts must connect in a closed circular arrangement to create voltage.
+The text also discusses formulating hypotheses using independent and dependent variables.</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -56601,7 +57409,12 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers topics in chemistry and physics.
+It discusses acids and bases, as well as electrical circuits.
+A simple electrical circuit requires a wire, battery, and bulb connected in series.
+Conductive parts must connect in a closed circular arrangement to create voltage.
+Hypothesis formulation and experimentation are also briefly introduced.</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -56634,7 +57447,12 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses acids, bases, and chemical reactions.
+It also covers electrical circuits and hypothesis formulation.
+A good hypothesis includes an independent and dependent variable.
+The text emphasizes that hypotheses may not be confirmed after experimentation.
+Scientific experiments can lead to valuable knowledge even if the hypothesis is rejected.</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -56667,7 +57485,12 @@
       <c r="E162" s="3" t="n"/>
       <c r="F162" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text covers various scientific topics, including geology and biology.
+It discusses the composition of marble and its reaction with acid.
+A hypothesis is defined as an "If...then..." statement with variables.
+The text also touches on experimental procedures and variable identification.
+Scientific experiments and hypothesis testing are emphasized throughout.</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -56700,7 +57523,12 @@
       <c r="E163" s="3" t="n"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers biology basics and scientific experimentation.
+It discusses forming hypotheses with independent and dependent variables.
+A good hypothesis uses an "If...then..." statement to link variables.
+Experimentation may lead to rejection of a hypothesis, still providing valuable knowledge.
+The text also touches on electrical circuits and microscope images of lung cells.</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -56733,7 +57561,12 @@
       <c r="E164" s="3" t="n"/>
       <c r="F164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses basic biology concepts and definitions.
+It explores the diversity of organisms and cells that make up life.
+A hypothesis is introduced as a statement linking independent and dependent variables.
+The text explains how to formulate and test a hypothesis through experimentation.
+It emphasizes the importance of understanding variable relationships in scientific inquiry.</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -56766,7 +57599,12 @@
       <c r="E165" s="3" t="n"/>
       <c r="F165" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses cells and their diversity.
+It highlights the discovery of the nucleus in plant and animal cells, showing unity in life.
+A hypothesis is formulated with variables to test a theory.
+Experiments may confirm or reject a hypothesis, leading to valuable knowledge.
+The text guides readers through testing a hypothesis and analyzing experimental data.</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -56799,7 +57637,12 @@
       <c r="E166" s="3" t="n"/>
       <c r="F166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses cells, organisms, and biology concepts.
+It covers cell structures, including nuclei, organelles, and membranes.
+A hypothesis can be formulated to test relationships between variables.
+Experiments may confirm or reject hypotheses, leading to valuable knowledge.
+The text also guides readers through testing a hypothesis and analyzing results.</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -56836,7 +57679,12 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The discovery of the nucleus in cells reveals a unity in life.
+Plant and animal cells share common design and functions.
+The text describes cell components, including organelles and molecules.
+It also covers experimental procedures and variables in scientific investigations.
+Cell biology concepts are explained for middle school and high school students.</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -56873,7 +57721,11 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers cell biology for middle and high school students. 
+It discusses plant and animal cells, including organelles and their functions. 
+Key components like the nucleus, mitochondria, and cell membrane are highlighted. 
+The text also touches on experimental procedures and variables in cell biology experiments. 
+It provides an overview of cellular structure and function.</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -56906,7 +57758,11 @@
       <c r="E169" s="3" t="n"/>
       <c r="F169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers cell components and their importance. 
+It discusses the nucleus, mitochondria, and other organelles.
+The role of these components in biological development is highlighted.
+Experimental procedures and variables are also mentioned.
+Cell structure and function are the main themes.</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -56943,7 +57799,12 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The cell nucleus contains genetic material, namely DNA.
+Genes determine biological development and are inherited from parents.
+Characteristics pass from parent to child through genes in DNA.
+Cells have various components, including mitochondria and ribosomes.
+These components work together to support cellular function.</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -56976,7 +57837,11 @@
       <c r="E171" s="3" t="n"/>
       <c r="F171" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The cell nucleus is crucial as it contains genetic material, namely DNA. 
+Genes determine biological development and are inherited from parents. 
+Proteins and amino acids play a significant role in this process. 
+The cell's structure, including organelles, is essential for its function. 
+Genetic material is passed down through generations, influencing characteristics.</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -57009,7 +57874,12 @@
       <c r="E172" s="3" t="n"/>
       <c r="F172" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The cell contains genetic material, namely DNA, which passes characteristics from parent to child.
+Genes are specific parts of DNA that determine inherited traits.
+DNA is composed of nucleotides with four different nitrogen bases: A, T, C, and G.
+These bases pair in a complementary manner, forming a double-stranded chain.
+The text also covers cell structure, including organelles and proteins made from amino acid chains.</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -57042,7 +57912,12 @@
       <c r="E173" s="3" t="n"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers proteins, amino acids, and nucleic acids.
+It explains the structure of DNA and its building blocks, nucleotides.
+There are 20 amino acids and 4 types of nucleotides in DNA.
+The central doctrine of biology involves protein synthesis and genetic information flow.
+The text also touches on cell components and structures, including organelles and chromosomes.</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -57075,7 +57950,12 @@
       <c r="E174" s="3" t="n"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The structure of nucleic acids, specifically DNA, is composed of nucleotides.
+Nucleotides consist of a nitrogen base, sugar, and phosphate group.
+There are four types of nucleotides in DNA, differing only in their nitrogen base.
+The flow of genetic information is fundamental to molecular biology and genetics.
+Cellular components, including the nucleus and organelles, play a crucial role in this process.</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -57108,7 +57988,7 @@
       <c r="E175" s="3" t="n"/>
       <c r="F175" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers the central doctrine of biology, focusing on protein synthesis and genetic information. It introduces key cellular components and structures. The flow of genetic information is emphasized as a basis for molecular biology. The text invites readers to take on a researcher role and explore hypotheses. It provides an overview of cell structure and biology concepts.</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -57141,7 +58021,12 @@
       <c r="E176" s="3" t="n"/>
       <c r="F176" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+The text introduces a biology research scenario, exploring protein synthesis and DNA's role. 
+It invites readers to investigate cellular components and their functions. 
+Key topics include cell structure and biology concepts, such as mitochondria and ribosomes. 
+The text aims to engage readers in an interactive learning experience. 
+Cellular biology and investigation are the primary themes covered.</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -57174,7 +58059,12 @@
       <c r="E177" s="3" t="n"/>
       <c r="F177" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+The text explores the world of biology, focusing on cellular components.
+It invites investigation into DNA's role in protein synthesis.
+Key biological processes like replication, transcription, and translation are mentioned.
+Cellular structures such as mitochondria, ribosomes, and the nucleus are listed.
+The text appears to be an introduction to a biology-themed game or educational resource.</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -57207,7 +58097,12 @@
       <c r="E178" s="3" t="n"/>
       <c r="F178" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text explores protein synthesis and DNA's role in it.
+It investigates replication, transcription, and translation processes.
+Variations in DNA sequences and their effects on phenotypes are discussed.
+Cell structure components such as mitochondria and ribosomes are listed.
+The text appears to be an educational game or lesson on cell biology and genetics.</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -57240,7 +58135,12 @@
       <c r="E179" s="3" t="n"/>
       <c r="F179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses DNA, RNA, and protein synthesis.
+It covers transcription, translation, and replication processes.
+Variations in DNA sequences and their effects on phenotypes are explored.
+Cell structure and organelles, such as mitochondria and ribosomes, are mentioned.
+The text appears to be a study guide or educational resource for cell biology.</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -57273,7 +58173,11 @@
       <c r="E180" s="3" t="n"/>
       <c r="F180" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text explores DNA's role in transcription and translation. 
+It discusses how DNA variations affect phenotypes. 
+Cellular components are listed, including organelles and structures. 
+The process of protein generation is mentioned as complex. 
+Cell types, such as prokaryotic and eukaryotic cells, are referenced.</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -57306,7 +58210,12 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text explores DNA and its role in transcription and translation.
+It discusses how variations in DNA sequences produce different phenotypes.
+Population genetics studies genetic differences within and between populations.
+Evolutionary biology examines adaptation, speciation, and population structure.
+The study of evolution combines with genetics to understand changes in allele proportions over time.</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -57339,7 +58248,11 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers DNA, transcription, and translation.
+It explores variations in DNA sequences and their effects on phenotypes.
+Population genetics and evolutionary biology are also discussed.
+The role of natural selection and other mechanisms in evolution is examined.
+Evolutionary concepts are illustrated through simulation models and virtual experiments.</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -57372,7 +58285,11 @@
       <c r="E183" s="3" t="n"/>
       <c r="F183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Population genetics studies genetic differences within populations.
+It's a part of evolutionary biology, examining adaptation and speciation.
+The field combines evolutionary theory with genetics understanding.
+Simulations like the agent-based model help illustrate concepts.
+Evolution is defined as changes in allele proportions over time.</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -57405,7 +58322,12 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+Population genetics studies genetic differences within and between populations.
+It's a part of evolutionary biology, examining adaptation, speciation, and population structure.
+The text discusses Hardy-Weinberg theory and its assumptions, including small population, selection, mutation, and non-random mating.
+A simulation model is used to demonstrate microevolutionary processes, including genetic drift and natural selection.
+The model helps students understand complex concepts in evolutionary biology through virtual experiments.</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -57438,7 +58360,12 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses an agent-based population genetics simulation model.
+It explores microevolutionary processes, including natural selection and genetic drift.
+The model allows students to conduct virtual experiments and test hypotheses.
+It features tools to demonstrate Hardy-Weinberg theory and its assumptions.
+The simulation helps students understand evolutionary concepts through interactive and graphical results.</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -57471,7 +58398,12 @@
       <c r="E186" s="3" t="n"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses an agent-based population genetics simulation model.
+It explores concepts like Hardy-Weinberg theory, natural selection, and genetic drift.
+The model simulates microevolutionary processes with factors like population size and mutation.
+Students can use the model to develop and test hypotheses through virtual experiments.
+The simulation helps illustrate challenging evolutionary concepts in a biologically realistic way.</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -57504,7 +58436,12 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses evolutionary theory and population genetics.
+It introduces an agent-based simulation model to study genetic drift and selection.
+The model explores how random events affect allele proportions in small populations.
+The text also references real-world experiments, such as John Endler's guppy study, to illustrate variations in physical characteristics.
+These concepts are used to investigate the influence of variables on evolutionary changes.</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -57537,7 +58474,12 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses population genetics simulation and evolutionary theory.
+It introduces an agent-based model to conduct virtual experiments on Hardy-Weinberg theory assumptions.
+A case study on guppies and their varying physical characteristics is presented.
+The Sexual Selection in Guppies virtual laboratory allows users to run simulations to determine variables influencing spot variation.
+The goal is to understand the factors responsible for trends in spot numbers over time.</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -57570,7 +58512,12 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses population genetics and evolutionary theory.
+It introduces an agent-based simulation model and a virtual lab on guppy experiments.
+The goal is to investigate variables influencing physical characteristics, such as spots in male guppies.
+Sexual selection and other factors like mutation and migration are explored.
+The text also touches on real-world examples, including lice resistance to shampoo chemicals.</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -57603,7 +58550,12 @@
       <c r="E190" s="3" t="n"/>
       <c r="F190" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses evolutionary theory and population genetics.
+It explores natural selection and variation in species, such as guppies.
+Simulations and experiments are used to investigate factors influencing traits.
+Variables like environment, mutation, and selection are analyzed.
+The goal is to understand how these factors shape the evolution of species.</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -57636,7 +58588,11 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses population genetics simulations and evolutionary theory. 
+It explores natural selection through virtual experiments with bunnies. 
+Variables such as mutation, migration, and non-random mating are examined. 
+The text also touches on adaptation and advantageous traits in different environments. 
+Evolutionary changes, like fur color and tooth length, are used as examples.</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -57669,7 +58625,12 @@
       <c r="E192" s="3" t="n"/>
       <c r="F192" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text explores evolutionary theory and natural selection.
+It discusses physical characteristics and attraction in humans and animals.
+Virtual laboratory experiments with bunnies investigate environmental adaptations.
+The text also touches on the development of resistance in lice to shampoos.
+Evolutionary advantages and trait changes are key themes throughout.</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -57706,7 +58667,11 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores natural selection and evolution.
+It discusses bunnies adapting to environments through mutations.
+The connection between star lightness and age is also investigated.
+Resistant lice strains in the US are attributed to chemical shampoo use.
+Evolutionary advantages and trait changes are examined in various habitats.</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -57739,7 +58704,12 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text explores natural selection and evolution through examples with bunnies.
+It discusses adaptations such as fur color and teeth length in different environments.
+Two explanations are provided to explain these adaptations.
+The text also touches on the life cycle of stars and their connection to age and lightness.
+Finally, it introduces atoms as the basic units of matter and their importance for life processes.</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -57772,7 +58742,11 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text explores natural selection and evolution.
+It discusses the connection between stars' lightness and age.
+The topic then shifts to atoms, their importance, and structure.
+Investigations and worksheets are provided for further learning.
+The text concludes with a review of life processes and self-evaluation.</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -57805,7 +58779,11 @@
       <c r="E196" s="3" t="n"/>
       <c r="F196" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores the connection between stars and their ages. 
+It also discusses investigating the life of stars using worksheets.
+The topic then shifts to atoms, the basic units of matter.
+Atoms are crucial for life processes and evolution.
+The text concludes with a call for self-evaluation and review.</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -57838,7 +58816,12 @@
       <c r="E197" s="3" t="n"/>
       <c r="F197" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses investigating star life and atomic structure.
+It mentions using worksheets and apps to facilitate learning.
+Reflecting on time spent in different phases is also encouraged.
+The text then shifts to exploring atoms, their importance, and composition.
+The goal is to complete a tour of life processes and self-evaluate understanding.</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -57871,7 +58854,12 @@
       <c r="E198" s="3" t="n"/>
       <c r="F198" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses an Interactive Learning System (ILS) that tracks time spent on each phase.
+It provides tools to reflect on time management and phase switching.
+The system displays content from other apps and shows time spent on each activity.
+The topic shifts to atoms, their importance in life processes, and building atomic structures.
+The text concludes with a review and self-evaluation of the learning process.</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -57904,7 +58892,12 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses an Interactive Learning System (ILS) and its features.
+It tracks time spent on each phase and provides a chart for reflection.
+The ILS also explores scientific topics, such as atoms and life processes.
+A virtual laboratory on Sexual Selection in Guppies is introduced.
+Variables and their descriptions are provided for the virtual lab experiment.</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -57937,7 +58930,12 @@
       <c r="E200" s="3" t="n"/>
       <c r="F200" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers various topics including time management and phase tracking.
+It also touches on environmental changes and atomic structure.
+A tour of life processes is mentioned, with a call to review results.
+Sexual selection in guppies is another topic, with variables described.
+These themes seem unrelated, suggesting a collection of disparate ideas.</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -57974,7 +58972,12 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers various topics, including environmental changes and conservation. 
+It mentions a lake in Bolivia drying up due to environmental issues.
+A virtual laboratory on sexual selection in guppies is also discussed.
+Variables such as population size and predator numbers are considered.
+The text concludes with a prompt for self-evaluation and review.</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -58007,7 +59010,12 @@
       <c r="E202" s="3" t="n"/>
       <c r="F202" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses environmental changes and their impacts.
+Bolivia's second-largest lake is drying up, affecting Earth's water.
+A virtual lab on sexual selection in guppies is introduced.
+Variables such as population size and predator presence are considered.
+The text concludes with a prompt for self-evaluation.</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -58040,7 +59048,12 @@
       <c r="E203" s="3" t="n"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses environmental changes, such as a drying lake in Bolivia.
+It touches on impacts on water and icebergs.
+A virtual laboratory on sexual selection in guppies is also mentioned.
+Variables like population size and predator numbers are considered.
+The text appears to be a mix of ecology and biology topics.</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -58073,7 +59086,11 @@
       <c r="E204" s="3" t="n"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers climate trends and impacts on Earth. 
+It mentions temperature, carbon dioxide, and greenhouse gases. 
+A virtual lab on sexual selection in guppies is also discussed. 
+Variables such as population size and predator numbers are examined. 
+The text concludes with a call for self-evaluation and review.</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -58106,7 +59123,12 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+The text covers climate trends and impacts on Earth's water and ice. 
+It mentions historical temperature and greenhouse gas trends.
+A virtual lab on sexual selection in guppies is also described.
+Variables such as population size and predator numbers are discussed.
+Climate data visualization using graphs and plot menus is explained.</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -58139,7 +59161,12 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+The text discusses climate trends and impacts on Earth's water and ice. 
+It covers temperature, carbon dioxide, methane, and nitrous oxide levels.
+Historical data is explored over hundreds of thousands of years.
+Graphs are used to visualize the changing trends.
+The focus is on the last 5000 years, particularly the last 100 years.</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -58172,7 +59199,11 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text covers impacts of climate change on water and ice. 
+It explores historical climate trends over thousands of years. 
+Temperature, carbon dioxide, methane, and nitrous oxide levels are analyzed. 
+The relationship between climate change and greenhouse phenomena is discussed. 
+Climate trends are visualized through graphs and plots.</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -58209,7 +59240,11 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses climate change and its impacts.
+It explores historical climate trends over thousands of years.
+Key factors include temperature, carbon dioxide, methane, and nitrous oxide.
+The Greenhouse Effect is also examined in relation to climate change.
+Climate trends are visualized over the last 5000 years.</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -58242,7 +59277,12 @@
       <c r="E209" s="3" t="n"/>
       <c r="F209" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text explores historical climate trends over thousands of years.
+It covers temperature, carbon dioxide, methane, and nitrous oxide levels.
+Solar radiation's interaction with Earth's atmosphere causes global warming.
+Greenhouse gases like carbon dioxide contribute to the greenhouse effect.
+Climate change is linked to the greenhouse phenomenon.</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
@@ -58275,7 +59315,11 @@
       <c r="E210" s="3" t="n"/>
       <c r="F210" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text explores the interaction between solar radiation and the Earth's atmosphere.
+It discusses how greenhouse gases, such as carbon dioxide, affect the climate.
+The greenhouse effect and its impact on global warming are key topics.
+The role of atmospheric gases and clouds in climate change is also examined.
+The text aims to explain the scientific concepts of climate change.</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
@@ -58308,7 +59352,12 @@
       <c r="E211" s="3" t="n"/>
       <c r="F211" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+The text explores the interaction between solar radiation and the Earth's atmosphere, causing global warming.
+Greenhouse gases, such as carbon dioxide, play a significant role in the climate.
+The text also discusses the effects of clouds, glass panes, and atmospheric gases on the greenhouse effect.
+Simulations and experiments are used to understand and stabilize carbon output over time.
+The relationship between climate change and the greenhouse phenomenon is a central scientific concept.</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -58341,7 +59390,12 @@
       <c r="E212" s="3" t="n"/>
       <c r="F212" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text explores the impact of greenhouse gases on climate.
+It delves into the atmosphere's composition during the ice age and present day.
+The role of clouds, greenhouse gas concentration, and temperature changes are examined.
+The interaction between light and molecules is also discussed.
+The Greenhouse Effect and its relation to climate change are key themes.</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -58374,7 +59428,12 @@
       <c r="E213" s="3" t="n"/>
       <c r="F213" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+The text discusses climate change and carbon output.
+It explores strategies to stabilize carbon levels over 50 years.
+The role of greenhouse gases like CO2, methane, and nitrous oxide is examined.
+The interaction between IR photons and these gases is also studied.
+Climate change and the Greenhouse Effect are key scientific concepts covered.</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -58407,7 +59466,11 @@
       <c r="E214" s="3" t="n"/>
       <c r="F214" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text explores the absorption of infrared radiation by CO2.
+It illustrates energy transfer to surrounding molecules, affecting temperature.
+The animation demonstrates vibrational modes of CO2 and temperature rise.
+Climate change and the greenhouse effect are key scientific concepts discussed.
+The relationship between greenhouse phenomena and climate change is examined.</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -58440,7 +59503,11 @@
       <c r="E215" s="3" t="n"/>
       <c r="F215" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores ocean acidification and its impacts.
+It delves into climate change and the greenhouse effect.
+Greenhouse gases like CO2, N2O, and methane are discussed.
+The relationship between these gases and temperature is analyzed.
+Climate change concepts are examined through interactive models.</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -58473,7 +59540,11 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores ocean acidification and its impacts on sea life.
+It discusses climate change and the greenhouse effect.
+Up to 40% of manmade CO2 is captured by oceans, making them a significant carbon sink.
+However, this comes at a cost, as CO2 dissolves in water, increasing acidity.
+Ocean acidification affects marine life, particularly shell-forming organisms like sea urchin larvae.</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -58506,7 +59577,12 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text explores ocean acidification and its effects on sea life.
+It discusses the Greenhouse Effect and carbon sinks, including oceans.
+Up to 40% of manmade CO2 is captured by oceans, causing acidification.
+This acidification hinders carbonate formation and dissolves exoskeletons.
+The text also mentions interactive models and graph adjustments for climate variables.</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -58539,7 +59615,11 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text explores ocean acidification and its impacts on marine life.
+It discusses how oceans absorb CO2, becoming a significant carbon sink.
+However, this absorption comes with a cost, making the water more acidic.
+The chemistry of ocean acidification is explained through three chemical reactions.
+This affects the formation of carbonate compounds and can dissolve existing exoskeletons.</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -58572,7 +59652,11 @@
       <c r="E219" s="3" t="n"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores ocean acidification and its impacts on marine life. 
+Up to 40% of manmade CO2 is captured by oceans, rivers, and lakes. 
+This absorption changes water chemistry, making it more acidic. 
+Acidification hinders carbonate formation and can dissolve exoskeletons. 
+The text also discusses modeling climate variables like temperature and CO2 concentration.</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -58605,7 +59689,12 @@
       <c r="E220" s="3" t="n"/>
       <c r="F220" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers ocean acidification, plate tectonics, and climate change.
+It explores the chemistry of ocean acidification and its impacts on sea life.
+Up to 40% of manmade CO2 is captured by oceans, causing acidification.
+This process affects marine ecosystems and can dissolve existing exoskeletons.
+The text also discusses modeling climate change using graphs and variables.</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -58638,7 +59727,12 @@
       <c r="E221" s="3" t="n"/>
       <c r="F221" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+The text covers plate tectonics, continental drift, and carbon capture.
+It explains how oceans absorb CO2, becoming more acidic in the process.
+This acidification affects marine life and carbonate formation.
+The text also includes instructions for graphing CO2 emissions and temperature changes.
+Key variables include CO2 production, maximum temperature, and climate variability.</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -58671,7 +59765,12 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses plate tectonics and continental drift.
+It mentions a documentary on the subject by Isaac Frame.
+The topic also covers climate change and CO2 emissions.
+Graphs are used to illustrate temperature, CO2 concentration, and emission rates.
+Geologists concluded that the Earth's lithosphere is broken into moving plates.</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -58704,7 +59803,12 @@
       <c r="E223" s="3" t="n"/>
       <c r="F223" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+The documentary explores plate tectonics and continental drift.
+It covers processes like subduction and transduction, explaining how continents formed.
+Greece's location on the tectonic plate map is also examined.
+The text also touches on climate change, CO2 emissions, and temperature variability.
+Plate tectonics reveals the Earth's lithosphere is broken into moving plates.</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -58737,7 +59841,12 @@
       <c r="E224" s="3" t="n"/>
       <c r="F224" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text discusses tectonic plates and their motion.
+It mentions the division of the Earth's surface into plates, including Greece's location.
+The text also touches on climate change variables like CO2 emission rates and temperature.
+Geologists concluded that the Earth's lithosphere is broken into moving plates.
+This concept was established in the 1960s with around 12 large plates identified.</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -58774,7 +59883,12 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text discusses tectonic plates and their movement.
+It mentions Greece's location on the map of tectonic plates.
+Earthquake activity and climate variability are also touched upon.
+The text references CO2 production, temperature, and emissions rates.
+Geologists' conclusions about the Earth's lithosphere are mentioned.</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -58807,7 +59921,12 @@
       <c r="E226" s="3" t="n"/>
       <c r="F226" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses tectonic plates and earthquake activity.
+It also touches on climate change and CO2 production.
+Geologists have identified 12 large moving plates in the Earth's lithosphere.
+These plates are responsible for earthquake activity, including the "Ring of Fire".
+The text combines geology and climate change topics.</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -58840,7 +59959,12 @@
       <c r="E227" s="3" t="n"/>
       <c r="F227" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text discusses earthquake activity and data access.
+It also touches on climate change, CO2 production, and temperature variability.
+Geologists' findings on the Earth's lithosphere and moving plates are mentioned.
+The "Ring of Fire" and various tectonic plates are referenced.
+Earthquake and climate data are interconnected topics.</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -58873,7 +59997,12 @@
       <c r="E228" s="3" t="n"/>
       <c r="F228" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers earthquake data and climate change topics. 
+It mentions CO2 production, temperature, and climate variability.
+Geologists discovered the Earth's lithosphere is broken into moving plates.
+The "Ring of Fire" and various tectonic plates are mentioned.
+Earthquake and climate data are provided for analysis and self-assessment.</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -58906,7 +60035,12 @@
       <c r="E229" s="3" t="n"/>
       <c r="F229" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers earthquakes, climate data, and geology. 
+It mentions CO2 production, temperature, and climate variability.
+Geologists discovered the Earth's lithosphere is broken into moving plates.
+The text references the "Ring of Fire" and various tectonic plates.
+It appears to be a collection of notes on earth sciences and inquiry learning.</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -58939,7 +60073,12 @@
       <c r="E230" s="3" t="n"/>
       <c r="F230" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text covers various topics, including inquiry learning and Cymatics.
+Cymatics is the science of visualizing audio frequencies through music and science.
+Climate change is also discussed with statistics on CO2 production and temperature.
+Geology is mentioned, highlighting the Earth's lithosphere broken into moving plates.
+These topics seem unrelated, suggesting a collection of notes or resources.</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -58976,7 +60115,12 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text explores Cymatics, the science of visualizing audio frequencies.
+A video showcases enthusiastic individuals connecting music and science.
+The experiment uses a Tesla Coil and Plasma Ball to create visual effects.
+The text also briefly mentions plate tectonics and the Earth's lithosphere.
+It highlights an inspiring project that combines art and science.</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -59009,7 +60153,12 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text introduces Cymatics, the science of visualizing audio frequencies.
+A video showcases enthusiasts connecting music and science through innovative experiments.
+The experiments involve acoustics, electromagnetism, and waves, with some parts being real and others added for effect.
+The text warns against trying the experiments at home due to safety concerns.
+The topic will be explored further, starting from the basics of the scientific concepts involved.</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -59042,7 +60191,11 @@
       <c r="E233" s="3" t="n"/>
       <c r="F233" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores Cymatics, a science that visualizes audio frequencies. 
+It features a video showing music and science connection through experiments.
+These experiments involve sound waves, acoustics, and electromagnetism.
+They are presented in an innovative way, combining real experiments with special effects.
+The text warns against trying these experiments at home due to potential risks.</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -59075,7 +60228,11 @@
       <c r="E234" s="3" t="n"/>
       <c r="F234" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses sound waves and their properties. 
+It covers simple and complex sounds, wave forms, and frequencies. 
+Experiments with Tesla Coils and Plasma Balls are mentioned. 
+The text also touches on scientific concepts like acoustics and electromagnetism. 
+It highlights the innovative use of scientific facts in a video.</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -59108,7 +60265,12 @@
       <c r="E235" s="3" t="n"/>
       <c r="F235" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses sound and waves, covering topics like frequency and amplitude.
+It explains simple and complex sound waves, as well as transverse and longitudinal waves.
+Waves are defined by quantities such as wavelength, period, and velocity.
+These quantities are related to each other and affect the behavior of waves.
+The text also touches on scientific experiments and innovations related to acoustics and electromagnetism.</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -59141,7 +60303,12 @@
       <c r="E236" s="3" t="n"/>
       <c r="F236" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary of the text:
+The text discusses types of waves, including transverse and longitudinal waves.
+It covers wave properties such as amplitude, frequency, wavelength, and velocity.
+Mechanical waves are explored in detail, including reflection and superposition.
+Wave interference, including constructive and destructive interference, is also explained.
+The text combines scientific concepts with interactive simulations and experiments.</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -59174,7 +60341,12 @@
       <c r="E237" s="3" t="n"/>
       <c r="F237" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+Waves have properties like amplitude, frequency, wavelength, and velocity.
+These quantities are related to each other and affect wave behavior.
+Mechanical waves' velocity depends on their environment and wavelength.
+Wave phenomena include reflection, superposition, and interference.
+The text explores various scientific concepts related to acoustics and electromagnetism.</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -59207,7 +60379,12 @@
       <c r="E238" s="3" t="n"/>
       <c r="F238" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text explores mechanical waves and phenomena like reflection and superposition.
+It discusses wave interference, including constructive and destructive interference.
+The topics are related to acoustics, electromagnetism, and wave propagation.
+Experiments with sound waves and Ruben's Tube are mentioned as examples.
+The text aims to explain the science behind innovative experiments with waves.</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -59240,7 +60417,11 @@
       <c r="E239" s="3" t="n"/>
       <c r="F239" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores scientific phenomena used in innovative experiments. 
+It mentions Ruben's Tube and acoustic effects.
+Experiments involve acoustics, electromagnetism, and wave dynamics.
+Scientific facts are presented in an engaging and creative way.
+The video features real experiments and added visual effects.</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -59273,7 +60454,12 @@
       <c r="E240" s="3" t="n"/>
       <c r="F240" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text discusses Ruben's Tube and its creation.
+It involves scientific phenomena like acoustics and electromagnetism.
+Experiments with sound waves and fluid dynamics are showcased.
+The video features innovative uses of scientific facts and real experiments.
+The topic explores the intersection of sound, light, and physics.</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -59306,7 +60492,11 @@
       <c r="E241" s="3" t="n"/>
       <c r="F241" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses a video featuring innovative scientific experiments. 
+Experiments involve acoustics, electromagnetism, and waves.
+They include fluid dynamics and Tesla coils.
+Some parts are real, while others are added effects.
+The video showcases unique applications of scientific concepts.</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -59339,7 +60529,11 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses innovative scientific experiments with fluids and sound.
+It explores concepts related to acoustics, electromagnetism, and waves.
+Experiments include Ruben's Tube and Tesla coil demonstrations.
+These experiments are used to explain scientific facts in an engaging way.
+The text aims to educate on various scientific principles.</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -59372,7 +60566,11 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses scientific concepts related to acoustics and waves.
+Experiments are used to demonstrate innovative ideas and effects.
+Density is a key topic, explaining why objects sink or float.
+The text warns against attempting experiments at home.
+Scientific facts are presented in an engaging and educational way.</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -59405,7 +60603,12 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text explores concepts of sinking and floating.
+It introduces the concept of density and its relation to weight and size.
+Density is measured in grams per cubic centimeter, combining mass and volume.
+A higher density indicates that an object is heavier for its size.
+The text aims to help learners understand why objects sink or float based on their density.</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -59438,7 +60641,12 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses sinking and floating concepts.
+It introduces density as a key factor in determining if an object sinks or floats.
+Density is measured by weight (mass) and size (volume).
+Different materials have unique densities, affecting their buoyancy.
+Understanding density is crucial for designing good experiments.</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -59471,7 +60679,11 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text covers concepts of density and volume. 
+Density is measured in grams per cubic cm, indicating an object's weight and size. 
+A higher density means an object is heavier for its size. 
+The text also introduces experimentation and critical reflection. 
+It discusses designing good experiments, using an example of baking a cake.</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -59504,7 +60716,11 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses designing good experiments. 
+A good experiment involves changing one variable at a time. 
+This approach helps identify cause-and-effect relationships. 
+Changing multiple variables can lead to unclear results. 
+Only varying one thing at a time is key to a successful experiment.</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -59537,7 +60753,11 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses designing a good experiment by changing one variable at a time. 
+It uses baking a cake as an example to illustrate this concept.
+The goal is to identify cause-and-effect relationships.
+Changing multiple variables can lead to unclear results.
+A good experiment tests to falsify a hypothesis, not prove it right.</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -59570,7 +60790,11 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses the principles of designing a good experiment. 
+It emphasizes the importance of varying one thing at a time. 
+This approach helps to identify cause-and-effect relationships.
+A good experiment should test hypotheses, not prove them right.
+It applies these principles to evaluate experiments by Anna and Simon.</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -59603,7 +60827,12 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+The text discusses experimental design and the importance of testing hypotheses.
+It highlights common pitfalls, such as trying to prove oneself right.
+A key concept is "falsify," or testing if one is wrong.
+Anna's experiment is critiqued for its flaws in designing a good test.
+Good experimentation involves objective testing and variable manipulation.</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -59636,7 +60865,12 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text explores concepts of buoyancy and density.
+Anna conducts experiments changing mass, volume, and density.
+Her goal is to make objects float, but her experiment has flaws.
+Simon also explores buoyancy, believing heavy objects sink faster.
+The exercises aim to understand the relationship between density and buoyancy.</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -59669,7 +60903,11 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses concepts related to physics and experimentation.
+It touches on ideas about mass, volume, and density.
+A character named Simon conducts experiments to test his theory about sinking objects.
+His experiments involve changing the mass, volume, and density of objects.
+The text questions the validity of Simon's experimental approach.</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -59702,7 +60940,11 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses experiments on sinking objects and density.
+Simon tests how mass, volume, and density affect an object's ability to sink.
+He conducts three experiments with varying masses and volumes but constant density.
+The experiments are deemed not very good, prompting questions about their flaws.
+Improving the experiment design is suggested as a next step.</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -59735,7 +60977,11 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses experiments with density and buoyancy.
+It highlights flaws in previous experiments by others.
+A new investigation is proposed to explore what makes objects sink.
+Density is suspected as the key factor.
+The goal is to design better experiments to test this hypothesis.</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -59768,7 +61014,12 @@
       <c r="E255" s="3" t="n"/>
       <c r="F255" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses CERN and its collider.
+It introduces experiments on density and volume.
+The experiments have flaws, making them "not very good".
+Readers are prompted to design their own investigation.
+The goal is to explore what causes objects to sink or float based on density.</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -59801,7 +61052,12 @@
       <c r="E256" s="3" t="n"/>
       <c r="F256" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses CERN and its purpose in nuclear research.
+It explains the structure of matter at smaller scales, from atoms to quarks.
+The Standard Model governs interactions between basic building blocks of matter.
+Experiments on density are presented, with flaws identified.
+The reader is invited to design their own investigation on object density.</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -59834,7 +61090,12 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses CERN, a European nuclear research organization.
+It introduces the concept of the Large Hadron Collider and its purpose.
+The Standard Model explains how matter interacts through fundamental forces.
+An experiment investigating object density and sinking is proposed.
+The text encourages readers to learn about CERN and conduct their own investigation.</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -59867,7 +61128,11 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses CERN and the Large Hadron Collider. 
+It explains the structure of matter and the Standard Model. 
+The text also introduces an experiment on density and object buoyancy. 
+Investigations and research are encouraged to understand physics concepts. 
+Key topics include particle physics, experimentation, and scientific inquiry.</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -59900,7 +61165,11 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses CERN and the Large Hadron Collider. 
+It explains the structure of matter and the Standard Model.
+The collider's purpose and main tasks are outlined.
+Potential applications in physics, biology, and medicine are explored.
+Risks and threats associated with the collider's work are also assessed.</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -59933,7 +61202,12 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses CERN and the Large Hadron Collider.
+It explains the structure of matter and the Standard Model.
+The collider's purpose and potential applications are explored.
+Risks and threats associated with the collider are also assessed.
+The text raises questions about the benefits and dangers of LHC-based research.</t>
         </is>
       </c>
     </row>
@@ -59961,7 +61235,12 @@
       <c r="E261" s="3" t="n"/>
       <c r="F261" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief summary:
+CERN's Large Hadron Collider is explained through interactive models and animations.
+The Standard Model of physics governs the basic building blocks of matter.
+Research applications include physics, biology, chemistry, and medicine.
+Risks and threats associated with the collider are assessed.
+Investment in LHC-based research is considered amidst its 10-year lifespan.</t>
         </is>
       </c>
     </row>
@@ -59989,7 +61268,11 @@
       <c r="E262" s="3" t="n"/>
       <c r="F262" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text explores the structure of matter at smaller scales.
+It introduces the Standard Model and fundamental forces governing interactions.
+The Large Hadron Collider (LHC) is discussed, including its operation and potential applications.
+Various "hats" represent different perspectives: optimistic (Yellow), critical (Black), and emotional (Red).
+The LHC's impact and future are considered, weighing risks and benefits.</t>
         </is>
       </c>
     </row>
@@ -60017,7 +61300,12 @@
       <c r="E263" s="3" t="n"/>
       <c r="F263" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses STEM education and research projects.
+Students investigate the Arctic Pole and climate change.
+They use various "hats" to approach problems, such as Green Hat for modification and Yellow Hat for optimism.
+Research topics include physics, biology, and the Large Hadron Collider.
+The goal is to promote interest in science, technology, engineering, and mathematics education.</t>
         </is>
       </c>
     </row>
@@ -60045,7 +61333,12 @@
       <c r="E264" s="3" t="n"/>
       <c r="F264" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text promotes STEM education, encouraging students to learn about science and climate change.
+Students investigate the Arctic Pole, its problems, and ways to prevent further climate change.
+The text also explores the applications of physics, biology, and chemistry in various fields.
+It discusses the Large Hadron Collider, its risks, and potential benefits.
+Overall, it aims to foster critical thinking and awareness about science and its implications.</t>
         </is>
       </c>
     </row>
@@ -60073,7 +61366,12 @@
       <c r="E265" s="3" t="n"/>
       <c r="F265" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a brief 5-line summary:
+The text promotes STEM education and encourages students to learn about the Arctic Pole.
+Students investigate climate changes and their consequences in the Arctic region.
+Objectives include learning about the Arctic Pole, understanding climate change, and finding prevention methods.
+The text also touches on critical thinking exercises using different colored hats to analyze problems.
+These exercises aim to develop research, risk assessment, and intuitive skills among students.</t>
         </is>
       </c>
     </row>
@@ -60101,7 +61399,11 @@
       <c r="E266" s="3" t="n"/>
       <c r="F266" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses critical thinking exercises using colored hats. 
+It involves analyzing information from a video and websites. 
+The colors represent different perspectives: white (facts), yellow (optimism), black (risks), and red (emotions). 
+These hats are used to evaluate topics like the Large Hadron Collider. 
+Critical thinking is applied to assess successes, risks, and emotions related to the topic.</t>
         </is>
       </c>
     </row>
@@ -60129,7 +61431,11 @@
       <c r="E267" s="3" t="n"/>
       <c r="F267" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses critical thinking exercises using different colored hats. 
+It covers research and analysis of successes and risks. 
+The Large Hadron Collider is used as a case study to assess benefits and threats. 
+Different perspectives, including optimistic and pessimistic views, are considered. 
+Critical thinking and evaluation of information are key themes.</t>
         </is>
       </c>
     </row>
@@ -60157,7 +61463,11 @@
       <c r="E268" s="3" t="n"/>
       <c r="F268" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text discusses critical thinking exercises using different colored hats. 
+Yellow hat focuses on successes and advantages.
+Black hat assesses risks and threats.
+Red hat considers emotions and intuition.
+The Large Hadron Collider is used as an example for these thought experiments.</t>
         </is>
       </c>
     </row>
@@ -60185,7 +61495,11 @@
       <c r="E269" s="3" t="n"/>
       <c r="F269" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>The text explores climate change and greenhouse gases.
+It discusses simulating the Greenhouse effect and atmospheric changes.
+The Large Hadron Collider is also mentioned, with its risks and benefits assessed.
+Applications of physics, biology, and chemistry are considered.
+The text invites experimentation and critical thinking about science and its implications.</t>
         </is>
       </c>
     </row>
@@ -60213,7 +61527,7 @@
       <c r="E270" s="3" t="n"/>
       <c r="F270" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text explores climate change and greenhouse effects through experiments and simulations. It discusses the impact of greenhouse gases on temperature and atmosphere. The text also touches on the applications of physics, biology, and chemistry in various fields. Additionally, it mentions the Large Hadron Collider and its potential risks and benefits. Overall, it covers science, technology, and environmental topics.</t>
         </is>
       </c>
     </row>
@@ -60241,7 +61555,12 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text covers various scientific topics, including climate change and greenhouse gases.
+It also touches on the Large Hadron Collider and its potential risks and benefits.
+Vaccinations are another topic, with discussions on herd immunity and disease prevention.
+The importance of high vaccination rates to protect vulnerable populations is highlighted.
+These topics are explored through experiments, simulations, and real-world examples.</t>
         </is>
       </c>
     </row>
@@ -60273,7 +61592,12 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses climate change and vaccinations.
+It explores the greenhouse effect and atmospheric gases.
+Vaccinations are also covered, including rotavirus and measles outbreaks.
+Herd immunity is mentioned as a key benefit of high vaccination rates.
+The text includes news articles and simulations related to these topics.</t>
         </is>
       </c>
     </row>
@@ -60305,7 +61629,11 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Vaccinations are increasingly available for various diseases. 
+Universal vaccination programs aim for high vaccination rates to protect all individuals.
+Herd immunity is achieved when a high percentage of the population is vaccinated.
+News articles highlight rotavirus vaccination results in India and a measles outbreak in New York.
+These examples illustrate the importance of vaccinations in preventing disease outbreaks.</t>
         </is>
       </c>
     </row>
@@ -60333,7 +61661,12 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses vaccinations and outbreaks.
+It mentions rotavirus and measles outbreaks in India and New York.
+The authors introduce an inquiry space on vaccines with limited immunity.
+They focus on the influenza vaccine, which doesn't provide lifelong immunity.
+The topic will explore a specific case related to the influenza vaccine.</t>
         </is>
       </c>
     </row>
@@ -60361,7 +61694,12 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief 5-line summary:
+The text discusses vaccination news and outbreaks.
+It mentions a measles outbreak in New York and rotavirus vaccination.
+The focus shifts to the influenza vaccine, which doesn't provide lifelong immunity.
+A specific case is examined: influenza vaccination for healthcare workers (HCW).
+This case highlights the impact of high influenza rates on hospital resources.</t>
         </is>
       </c>
     </row>
@@ -60393,7 +61731,12 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a brief summary:
+The text discusses vaccination news and outbreaks.
+It focuses on the influenza vaccine, which doesn't provide lifelong immunity.
+A specific case examines influenza vaccination for healthcare workers (HCW).
+In 2018, high influenza rates affected hospitals' resources and personnel.
+Hospitals were overwhelmed, with some treating patients in tents.</t>
         </is>
       </c>
     </row>
@@ -60421,7 +61764,12 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses recent outbreaks and vaccination news.
+It highlights the challenges faced during the 2017-2018 influenza season.
+Hospitals were overwhelmed, with some forced to postpone operations or close ERs.
+Influenza vaccinations are crucial, especially for healthcare workers.
+Vaccination of healthcare workers is a key topic due to their high risk of infection.</t>
         </is>
       </c>
     </row>
@@ -60449,7 +61797,12 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses various vaccination news and outbreaks.
+It highlights the challenges faced during the 2017-2018 influenza season.
+Influenza vaccinations are needed annually due to constantly changing viruses.
+Healthcare workers are at risk of contracting influenza, putting patients at greater risk.
+Vaccination for healthcare workers is a crucial topic to investigate and consider.</t>
         </is>
       </c>
     </row>
@@ -60477,7 +61830,12 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary of the text:
+The text discusses vaccination and prevention of diseases like rotavirus, measles, and influenza.
+Influenza vaccines must be given annually due to constantly changing virus types.
+Healthcare workers are at risk of contracting influenza, with 25% of hospital-infected patients dying.
+Vaccination of healthcare workers is a crucial topic, especially after seasons with high influenza rates.
+The debate centers around whether healthcare workers should get vaccinated for influenza every year.</t>
         </is>
       </c>
     </row>
@@ -60505,7 +61863,12 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+The text discusses vaccination news and outbreaks.
+It mentions rotavirus, measles, and influenza seasons.
+Healthcare workers' vaccination habits are questioned.
+Some workers claim vaccinations are ineffective due to past experiences.
+The text invites investigation into vaccine effectiveness.</t>
         </is>
       </c>
     </row>
@@ -60533,7 +61896,11 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>The text discusses vaccination news and influenza season updates. 
+It explores reasons healthcare workers decline flu vaccinations, including ineffective past vaccinations.
+A interactive graph is introduced to analyze vaccination effectiveness.
+Variables such as vaccination rates and illness percentages are considered.
+The goal is to investigate the benefits of influenza vaccination for healthcare workers.</t>
         </is>
       </c>
     </row>
@@ -60561,7 +61928,12 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Here is a 5-line summary:
+The text discusses vaccination news and outbreaks.
+It mentions rotavirus, measles, and influenza season updates.
+An interactive graph is introduced to investigate vaccination effects.
+The graph tracks variables such as vaccinated healthcare workers and influenza cases.
+The goal is to analyze the impact of vaccination on preventing illnesses.</t>
         </is>
       </c>
     </row>
@@ -60589,7 +61961,12 @@
       <c r="E283" s="3" t="n"/>
       <c r="F283" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+Measles outbreak in New York sparks investigation.
+Influenza season news requires analysis using interactive graphs.
+Variables include vaccination rates and illness cases among healthcare workers (HCW).
+Graphs track ILIs, influenza, and prevented cases based on vaccination rates.
+Investigation guidelines provide support for understanding the data.</t>
         </is>
       </c>
     </row>
@@ -60617,7 +61994,12 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Here is a 5-line summary:
+A measles outbreak in New York and influenza season news are discussed.
+An interactive graph investigates identified cases and vaccination effectiveness.
+The graph tracks healthcare worker (HCW) vaccination rates and illness incidence.
+Variables include vaccination percentage, confirmed influenza, and prevented cases.
+Users can explore different scenarios by adjusting severity and vaccination quality.</t>
         </is>
       </c>
     </row>

</xml_diff>